<commit_message>
Updated schedule template to enable testing
</commit_message>
<xml_diff>
--- a/templates/schedule_pask.xlsx
+++ b/templates/schedule_pask.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ulfhk\Documents\Svenska Kyrkan\Kyrkan aktuell\0. Events\Click n Collect\Påskmarknad\2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atw10wp4\JupyterLab\Kyrkan\WebShopReport\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C344A019-C589-4CD1-B18F-F7F7B2B067E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70049E4C-ABF8-4E72-B4E7-2BA98CE31369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schema" sheetId="9" r:id="rId1"/>
@@ -18,9 +18,9 @@
   </sheets>
   <definedNames>
     <definedName name="DB_Dagar">Schema!#REF!</definedName>
-    <definedName name="DB_DagLista">Schema!$A$3:$A$42</definedName>
+    <definedName name="DB_DagLista">Schema!$A$2:$A$40</definedName>
     <definedName name="DB_Kalender">Schema!#REF!</definedName>
-    <definedName name="DB_Schema">Schema!$A$3:$B$42</definedName>
+    <definedName name="DB_Schema">Schema!$A$2:$B$40</definedName>
     <definedName name="DB_Slots">Schema!#REF!</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">Dag_Mall!$2:$2</definedName>
   </definedNames>
@@ -86,7 +86,7 @@
     <numFmt numFmtId="165" formatCode="_-[$€-C07]\ * #,##0.00_-;\-[$€-C07]\ * #,##0.00_-;_-[$€-C07]\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy;@"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -526,13 +526,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{463EB100-D71F-4CB0-A8C4-FF87F19718DC}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:B38"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <dimension ref="A1:B36"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="12.28515625" customWidth="1"/>
+    <col min="1" max="2" width="12.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -540,299 +540,283 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="6">
-        <v>45751</v>
+        <v>46102</v>
       </c>
       <c r="B2" s="14">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>0.54166666666666663</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="6">
-        <v>45752</v>
+        <v>46102</v>
       </c>
       <c r="B3" s="14">
+        <v>0.55555555555555547</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B4" s="14">
+        <v>0.5625</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B5" s="14">
+        <v>0.56944444444444431</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B6" s="14">
+        <v>0.58333333333333315</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B7" s="14">
+        <v>0.59722222222222199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B8" s="14">
+        <v>0.61111111111111083</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B9" s="14">
+        <v>0.62499999999999967</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B10" s="14">
+        <v>0.63888888888888851</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B11" s="14">
+        <v>0.65277777777777735</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B12" s="14">
+        <v>0.66666666666666619</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B13" s="14">
+        <v>0.68055555555555503</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="6">
+        <v>46102</v>
+      </c>
+      <c r="B14" s="14">
+        <v>0.69444444444444386</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B15" s="14">
         <v>0.54166666666666663</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B4" s="14">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B16" s="14">
         <v>0.55555555555555547</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B5" s="14">
-        <v>0.5625</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B6" s="14">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B17" s="14">
         <v>0.56944444444444431</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B7" s="14">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B18" s="14">
         <v>0.58333333333333315</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B8" s="14">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B19" s="14">
         <v>0.59722222222222199</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B9" s="14">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B20" s="14">
         <v>0.61111111111111083</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B10" s="14">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B21" s="14">
         <v>0.62499999999999967</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B11" s="14">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B22" s="14">
         <v>0.63888888888888851</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B12" s="14">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B23" s="14">
         <v>0.65277777777777735</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B13" s="14">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B24" s="14">
         <v>0.66666666666666619</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B14" s="14">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B25" s="14">
         <v>0.68055555555555503</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="6">
-        <v>45752</v>
-      </c>
-      <c r="B15" s="14">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="6">
+        <v>46103</v>
+      </c>
+      <c r="B26" s="14">
         <v>0.69444444444444386</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B16" s="14">
-        <v>0.54166666666666663</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B17" s="14">
-        <v>0.55555555555555547</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B18" s="14">
-        <v>0.56944444444444431</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B19" s="14">
-        <v>0.58333333333333315</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B20" s="14">
-        <v>0.59722222222222199</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B21" s="14">
-        <v>0.61111111111111083</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B22" s="14">
-        <v>0.62499999999999967</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B23" s="14">
-        <v>0.63888888888888851</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B24" s="14">
-        <v>0.65277777777777735</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
-      <c r="A25" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B25" s="14">
-        <v>0.66666666666666619</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2">
-      <c r="A26" s="6">
-        <v>45753</v>
-      </c>
-      <c r="B26" s="14">
-        <v>0.68055555555555503</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="6">
-        <v>45753</v>
+        <v>46104</v>
       </c>
       <c r="B27" s="14">
-        <v>0.69444444444444386</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="6">
-        <v>45754</v>
+        <v>46104</v>
       </c>
       <c r="B28" s="14">
-        <v>0.625</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2">
+        <v>0.63888888888888884</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="6">
-        <v>45754</v>
+        <v>46104</v>
       </c>
       <c r="B29" s="14">
-        <v>0.63888888888888884</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2">
+        <v>0.65277777777777768</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="6">
-        <v>45754</v>
+        <v>46104</v>
       </c>
       <c r="B30" s="14">
-        <v>0.65277777777777768</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2">
+        <v>0.66666666666666652</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="6">
-        <v>45754</v>
+        <v>46104</v>
       </c>
       <c r="B31" s="14">
-        <v>0.66666666666666652</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
+        <v>0.68055555555555536</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="6">
-        <v>45754</v>
+        <v>46104</v>
       </c>
       <c r="B32" s="14">
-        <v>0.68055555555555536</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2">
+        <v>0.6944444444444442</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" s="6">
-        <v>45754</v>
+        <v>46104</v>
       </c>
       <c r="B33" s="14">
-        <v>0.6944444444444442</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2">
+        <v>0.70833333333333304</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="6">
-        <v>45754</v>
+        <v>46104</v>
       </c>
       <c r="B34" s="14">
-        <v>0.70833333333333304</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2">
+        <v>0.72222222222222188</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" s="6">
-        <v>45754</v>
+        <v>46104</v>
       </c>
       <c r="B35" s="14">
-        <v>0.72222222222222188</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2">
+        <v>0.73611111111111072</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" s="6">
-        <v>45754</v>
+        <v>46143</v>
       </c>
       <c r="B36" s="14">
-        <v>0.73611111111111072</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2">
-      <c r="A37" s="6">
-        <v>45756</v>
-      </c>
-      <c r="B37" s="14">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2">
-      <c r="A38" s="6">
-        <v>45778</v>
-      </c>
-      <c r="B38" s="14">
         <v>0.25</v>
       </c>
     </row>
@@ -848,18 +832,18 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I445"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="3.42578125" customWidth="1"/>
+    <col min="1" max="2" width="3.453125" customWidth="1"/>
     <col min="4" max="4" width="32" customWidth="1"/>
-    <col min="5" max="5" width="25.28515625" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.26953125" customWidth="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="39" customWidth="1"/>
-    <col min="8" max="8" width="17.28515625" customWidth="1"/>
+    <col min="8" max="8" width="17.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="9.6" customHeight="1"/>
-    <row r="2" spans="1:9" ht="27" customHeight="1">
+    <row r="1" spans="1:9" ht="9.65" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B2" s="2" t="e">
         <f>Schema!#REF!</f>
         <v>#REF!</v>
@@ -878,10 +862,10 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="E3" s="16"/>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B4" s="21">
         <v>6</v>
       </c>
@@ -901,7 +885,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="30" customHeight="1">
+    <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="15"/>
       <c r="B5" s="22"/>
       <c r="C5" s="22">
@@ -909,7 +893,7 @@
       </c>
       <c r="F5" s="9"/>
     </row>
-    <row r="6" spans="1:9" ht="30" customHeight="1">
+    <row r="6" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="20">
         <v>1</v>
       </c>
@@ -920,7 +904,7 @@
       <c r="G6" s="5"/>
       <c r="I6" s="8"/>
     </row>
-    <row r="7" spans="1:9" ht="30" customHeight="1">
+    <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="20">
         <v>2</v>
       </c>
@@ -931,7 +915,7 @@
       <c r="G7" s="5"/>
       <c r="I7" s="8"/>
     </row>
-    <row r="8" spans="1:9" ht="30" customHeight="1">
+    <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="20">
         <v>3</v>
       </c>
@@ -942,7 +926,7 @@
       <c r="G8" s="5"/>
       <c r="I8" s="8"/>
     </row>
-    <row r="9" spans="1:9" ht="30" customHeight="1">
+    <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="20">
         <v>4</v>
       </c>
@@ -953,7 +937,7 @@
       <c r="G9" s="5"/>
       <c r="I9" s="8"/>
     </row>
-    <row r="10" spans="1:9" ht="30" customHeight="1">
+    <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="20">
         <v>5</v>
       </c>
@@ -964,7 +948,7 @@
       <c r="G10" s="5"/>
       <c r="I10" s="8"/>
     </row>
-    <row r="11" spans="1:9" ht="30" customHeight="1">
+    <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="20">
         <v>6</v>
       </c>
@@ -975,7 +959,7 @@
       <c r="G11" s="5"/>
       <c r="I11" s="8"/>
     </row>
-    <row r="12" spans="1:9" ht="30" customHeight="1">
+    <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="20">
         <v>7</v>
       </c>
@@ -986,7 +970,7 @@
       <c r="G12" s="5"/>
       <c r="I12" s="8"/>
     </row>
-    <row r="13" spans="1:9" ht="30" customHeight="1">
+    <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="20">
         <v>8</v>
       </c>
@@ -997,7 +981,7 @@
       <c r="G13" s="5"/>
       <c r="I13" s="8"/>
     </row>
-    <row r="14" spans="1:9" ht="30" customHeight="1">
+    <row r="14" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="20">
         <v>9</v>
       </c>
@@ -1008,7 +992,7 @@
       <c r="G14" s="5"/>
       <c r="I14" s="8"/>
     </row>
-    <row r="15" spans="1:9" ht="30" customHeight="1">
+    <row r="15" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="20">
         <v>10</v>
       </c>
@@ -1019,7 +1003,7 @@
       <c r="G15" s="5"/>
       <c r="I15" s="8"/>
     </row>
-    <row r="16" spans="1:9" ht="30" customHeight="1">
+    <row r="16" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="20">
         <v>11</v>
       </c>
@@ -1030,7 +1014,7 @@
       <c r="G16" s="5"/>
       <c r="I16" s="8"/>
     </row>
-    <row r="17" spans="1:9" ht="30" customHeight="1">
+    <row r="17" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="20">
         <v>12</v>
       </c>
@@ -1041,7 +1025,7 @@
       <c r="G17" s="5"/>
       <c r="I17" s="8"/>
     </row>
-    <row r="18" spans="1:9" ht="30" customHeight="1">
+    <row r="18" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="20">
         <v>13</v>
       </c>
@@ -1052,7 +1036,7 @@
       <c r="G18" s="5"/>
       <c r="I18" s="8"/>
     </row>
-    <row r="19" spans="1:9" ht="30" customHeight="1">
+    <row r="19" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="20">
         <v>14</v>
       </c>
@@ -1063,7 +1047,7 @@
       <c r="G19" s="5"/>
       <c r="I19" s="8"/>
     </row>
-    <row r="20" spans="1:9" ht="30" customHeight="1">
+    <row r="20" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="20">
         <v>15</v>
       </c>
@@ -1074,7 +1058,7 @@
       <c r="G20" s="5"/>
       <c r="I20" s="8"/>
     </row>
-    <row r="21" spans="1:9" ht="30" customHeight="1">
+    <row r="21" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="20">
         <v>16</v>
       </c>
@@ -1085,7 +1069,7 @@
       <c r="G21" s="5"/>
       <c r="I21" s="8"/>
     </row>
-    <row r="22" spans="1:9" ht="30" customHeight="1">
+    <row r="22" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="20">
         <v>17</v>
       </c>
@@ -1096,7 +1080,7 @@
       <c r="G22" s="5"/>
       <c r="I22" s="8"/>
     </row>
-    <row r="23" spans="1:9" ht="30" customHeight="1">
+    <row r="23" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="20">
         <v>18</v>
       </c>
@@ -1107,7 +1091,7 @@
       <c r="G23" s="5"/>
       <c r="I23" s="8"/>
     </row>
-    <row r="24" spans="1:9" ht="30" customHeight="1">
+    <row r="24" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="20">
         <v>19</v>
       </c>
@@ -1118,7 +1102,7 @@
       <c r="G24" s="5"/>
       <c r="I24" s="8"/>
     </row>
-    <row r="25" spans="1:9" ht="30" customHeight="1">
+    <row r="25" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="20">
         <v>20</v>
       </c>
@@ -1132,13 +1116,13 @@
       </c>
       <c r="I25" s="8"/>
     </row>
-    <row r="26" spans="1:9" ht="30" customHeight="1">
+    <row r="26" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="19"/>
       <c r="E26" s="12"/>
       <c r="F26" s="13"/>
       <c r="I26" s="8"/>
     </row>
-    <row r="27" spans="1:9" ht="30" customHeight="1">
+    <row r="27" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="15">
         <v>2</v>
       </c>
@@ -1148,7 +1132,7 @@
       </c>
       <c r="F27" s="9"/>
     </row>
-    <row r="28" spans="1:9" ht="30" customHeight="1">
+    <row r="28" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="20">
         <v>1</v>
       </c>
@@ -1159,7 +1143,7 @@
       <c r="G28" s="5"/>
       <c r="I28" s="8"/>
     </row>
-    <row r="29" spans="1:9" ht="30" customHeight="1">
+    <row r="29" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="20">
         <v>2</v>
       </c>
@@ -1170,7 +1154,7 @@
       <c r="G29" s="5"/>
       <c r="I29" s="8"/>
     </row>
-    <row r="30" spans="1:9" ht="30" customHeight="1">
+    <row r="30" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="20">
         <v>3</v>
       </c>
@@ -1181,7 +1165,7 @@
       <c r="G30" s="5"/>
       <c r="I30" s="8"/>
     </row>
-    <row r="31" spans="1:9" ht="30" customHeight="1">
+    <row r="31" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="20">
         <v>4</v>
       </c>
@@ -1192,7 +1176,7 @@
       <c r="G31" s="5"/>
       <c r="I31" s="8"/>
     </row>
-    <row r="32" spans="1:9" ht="30" customHeight="1">
+    <row r="32" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="20">
         <v>5</v>
       </c>
@@ -1203,7 +1187,7 @@
       <c r="G32" s="5"/>
       <c r="H32" s="8"/>
     </row>
-    <row r="33" spans="2:9" ht="30" customHeight="1">
+    <row r="33" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="20">
         <v>6</v>
       </c>
@@ -1214,7 +1198,7 @@
       <c r="G33" s="5"/>
       <c r="H33" s="8"/>
     </row>
-    <row r="34" spans="2:9" ht="30" customHeight="1">
+    <row r="34" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="20">
         <v>7</v>
       </c>
@@ -1225,7 +1209,7 @@
       <c r="G34" s="5"/>
       <c r="H34" s="8"/>
     </row>
-    <row r="35" spans="2:9" ht="30" customHeight="1">
+    <row r="35" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="20">
         <v>8</v>
       </c>
@@ -1236,7 +1220,7 @@
       <c r="G35" s="5"/>
       <c r="H35" s="8"/>
     </row>
-    <row r="36" spans="2:9" ht="30" customHeight="1">
+    <row r="36" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="20">
         <v>9</v>
       </c>
@@ -1248,7 +1232,7 @@
       <c r="H36" s="8"/>
       <c r="I36" s="8"/>
     </row>
-    <row r="37" spans="2:9" ht="30" customHeight="1">
+    <row r="37" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="20">
         <v>10</v>
       </c>
@@ -1260,7 +1244,7 @@
       <c r="H37" s="8"/>
       <c r="I37" s="8"/>
     </row>
-    <row r="38" spans="2:9" ht="30" customHeight="1">
+    <row r="38" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="20">
         <v>11</v>
       </c>
@@ -1272,7 +1256,7 @@
       <c r="H38" s="8"/>
       <c r="I38" s="8"/>
     </row>
-    <row r="39" spans="2:9" ht="30" customHeight="1">
+    <row r="39" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="20">
         <v>12</v>
       </c>
@@ -1284,7 +1268,7 @@
       <c r="H39" s="8"/>
       <c r="I39" s="8"/>
     </row>
-    <row r="40" spans="2:9" ht="30" customHeight="1">
+    <row r="40" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="20">
         <v>13</v>
       </c>
@@ -1296,7 +1280,7 @@
       <c r="H40" s="8"/>
       <c r="I40" s="8"/>
     </row>
-    <row r="41" spans="2:9" ht="30" customHeight="1">
+    <row r="41" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="20">
         <v>14</v>
       </c>
@@ -1308,7 +1292,7 @@
       <c r="H41" s="8"/>
       <c r="I41" s="8"/>
     </row>
-    <row r="42" spans="2:9" ht="30" customHeight="1">
+    <row r="42" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="20">
         <v>15</v>
       </c>
@@ -1320,7 +1304,7 @@
       <c r="H42" s="8"/>
       <c r="I42" s="8"/>
     </row>
-    <row r="43" spans="2:9" ht="30" customHeight="1">
+    <row r="43" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B43" s="20">
         <v>16</v>
       </c>
@@ -1331,7 +1315,7 @@
       <c r="G43" s="5"/>
       <c r="H43" s="8"/>
     </row>
-    <row r="44" spans="2:9" ht="30" customHeight="1">
+    <row r="44" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B44" s="20">
         <v>17</v>
       </c>
@@ -1342,7 +1326,7 @@
       <c r="G44" s="5"/>
       <c r="H44" s="8"/>
     </row>
-    <row r="45" spans="2:9" ht="30" customHeight="1">
+    <row r="45" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="20">
         <v>18</v>
       </c>
@@ -1354,7 +1338,7 @@
       <c r="H45" s="8"/>
       <c r="I45" s="8"/>
     </row>
-    <row r="46" spans="2:9" ht="30" customHeight="1">
+    <row r="46" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B46" s="20">
         <v>19</v>
       </c>
@@ -1366,7 +1350,7 @@
       <c r="H46" s="8"/>
       <c r="I46" s="8"/>
     </row>
-    <row r="47" spans="2:9" ht="30" customHeight="1">
+    <row r="47" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B47" s="20">
         <v>20</v>
       </c>
@@ -1381,14 +1365,14 @@
       <c r="H47" s="8"/>
       <c r="I47" s="8"/>
     </row>
-    <row r="48" spans="2:9" ht="30" customHeight="1">
+    <row r="48" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B48" s="19"/>
       <c r="E48" s="12"/>
       <c r="F48" s="13"/>
       <c r="H48" s="8"/>
       <c r="I48" s="8"/>
     </row>
-    <row r="49" spans="1:9" ht="30" customHeight="1">
+    <row r="49" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="15">
         <v>3</v>
       </c>
@@ -1400,7 +1384,7 @@
       <c r="H49" s="8"/>
       <c r="I49" s="8"/>
     </row>
-    <row r="50" spans="1:9" ht="30" customHeight="1">
+    <row r="50" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="20">
         <v>1</v>
       </c>
@@ -1412,7 +1396,7 @@
       <c r="H50" s="8"/>
       <c r="I50" s="8"/>
     </row>
-    <row r="51" spans="1:9" ht="30" customHeight="1">
+    <row r="51" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B51" s="20">
         <v>2</v>
       </c>
@@ -1424,7 +1408,7 @@
       <c r="H51" s="8"/>
       <c r="I51" s="8"/>
     </row>
-    <row r="52" spans="1:9" ht="30" customHeight="1">
+    <row r="52" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B52" s="20">
         <v>3</v>
       </c>
@@ -1435,7 +1419,7 @@
       <c r="G52" s="5"/>
       <c r="H52" s="8"/>
     </row>
-    <row r="53" spans="1:9" ht="30" customHeight="1">
+    <row r="53" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B53" s="20">
         <v>4</v>
       </c>
@@ -1446,7 +1430,7 @@
       <c r="G53" s="5"/>
       <c r="H53" s="8"/>
     </row>
-    <row r="54" spans="1:9" ht="30" customHeight="1">
+    <row r="54" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B54" s="20">
         <v>5</v>
       </c>
@@ -1458,7 +1442,7 @@
       <c r="H54" s="8"/>
       <c r="I54" s="8"/>
     </row>
-    <row r="55" spans="1:9" ht="30" customHeight="1">
+    <row r="55" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B55" s="20">
         <v>6</v>
       </c>
@@ -1470,7 +1454,7 @@
       <c r="H55" s="8"/>
       <c r="I55" s="8"/>
     </row>
-    <row r="56" spans="1:9" ht="30" customHeight="1">
+    <row r="56" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B56" s="20">
         <v>7</v>
       </c>
@@ -1482,7 +1466,7 @@
       <c r="H56" s="8"/>
       <c r="I56" s="8"/>
     </row>
-    <row r="57" spans="1:9" ht="30" customHeight="1">
+    <row r="57" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B57" s="20">
         <v>8</v>
       </c>
@@ -1494,7 +1478,7 @@
       <c r="H57" s="8"/>
       <c r="I57" s="8"/>
     </row>
-    <row r="58" spans="1:9" ht="30" customHeight="1">
+    <row r="58" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B58" s="20">
         <v>9</v>
       </c>
@@ -1506,7 +1490,7 @@
       <c r="H58" s="8"/>
       <c r="I58" s="8"/>
     </row>
-    <row r="59" spans="1:9" ht="30" customHeight="1">
+    <row r="59" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B59" s="20">
         <v>10</v>
       </c>
@@ -1518,7 +1502,7 @@
       <c r="H59" s="8"/>
       <c r="I59" s="8"/>
     </row>
-    <row r="60" spans="1:9" ht="30" customHeight="1">
+    <row r="60" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B60" s="20">
         <v>11</v>
       </c>
@@ -1530,7 +1514,7 @@
       <c r="H60" s="8"/>
       <c r="I60" s="8"/>
     </row>
-    <row r="61" spans="1:9" ht="30" customHeight="1">
+    <row r="61" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B61" s="20">
         <v>12</v>
       </c>
@@ -1542,7 +1526,7 @@
       <c r="H61" s="8"/>
       <c r="I61" s="8"/>
     </row>
-    <row r="62" spans="1:9" ht="30" customHeight="1">
+    <row r="62" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B62" s="20">
         <v>13</v>
       </c>
@@ -1553,7 +1537,7 @@
       <c r="G62" s="5"/>
       <c r="H62" s="8"/>
     </row>
-    <row r="63" spans="1:9" ht="30" customHeight="1">
+    <row r="63" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B63" s="20">
         <v>14</v>
       </c>
@@ -1564,7 +1548,7 @@
       <c r="G63" s="5"/>
       <c r="H63" s="8"/>
     </row>
-    <row r="64" spans="1:9" ht="30" customHeight="1">
+    <row r="64" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B64" s="20">
         <v>15</v>
       </c>
@@ -1576,7 +1560,7 @@
       <c r="H64" s="8"/>
       <c r="I64" s="8"/>
     </row>
-    <row r="65" spans="1:9" ht="30" customHeight="1">
+    <row r="65" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B65" s="20">
         <v>16</v>
       </c>
@@ -1588,7 +1572,7 @@
       <c r="H65" s="8"/>
       <c r="I65" s="8"/>
     </row>
-    <row r="66" spans="1:9" ht="30" customHeight="1">
+    <row r="66" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B66" s="20">
         <v>17</v>
       </c>
@@ -1600,7 +1584,7 @@
       <c r="H66" s="8"/>
       <c r="I66" s="8"/>
     </row>
-    <row r="67" spans="1:9" ht="30" customHeight="1">
+    <row r="67" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B67" s="20">
         <v>18</v>
       </c>
@@ -1612,7 +1596,7 @@
       <c r="H67" s="8"/>
       <c r="I67" s="8"/>
     </row>
-    <row r="68" spans="1:9" ht="30" customHeight="1">
+    <row r="68" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B68" s="20">
         <v>19</v>
       </c>
@@ -1624,7 +1608,7 @@
       <c r="H68" s="8"/>
       <c r="I68" s="8"/>
     </row>
-    <row r="69" spans="1:9" ht="30" customHeight="1">
+    <row r="69" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B69" s="20">
         <v>20</v>
       </c>
@@ -1639,13 +1623,13 @@
       <c r="H69" s="8"/>
       <c r="I69" s="8"/>
     </row>
-    <row r="70" spans="1:9" ht="30" customHeight="1">
+    <row r="70" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B70" s="19"/>
       <c r="E70" s="12"/>
       <c r="F70" s="13"/>
       <c r="H70" s="8"/>
     </row>
-    <row r="71" spans="1:9" ht="30" customHeight="1">
+    <row r="71" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="15">
         <v>4</v>
       </c>
@@ -1656,7 +1640,7 @@
       <c r="F71" s="9"/>
       <c r="H71" s="8"/>
     </row>
-    <row r="72" spans="1:9" ht="30" customHeight="1">
+    <row r="72" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B72" s="20">
         <v>1</v>
       </c>
@@ -1668,7 +1652,7 @@
       <c r="H72" s="8"/>
       <c r="I72" s="8"/>
     </row>
-    <row r="73" spans="1:9" ht="30" customHeight="1">
+    <row r="73" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B73" s="20">
         <v>2</v>
       </c>
@@ -1680,7 +1664,7 @@
       <c r="H73" s="8"/>
       <c r="I73" s="8"/>
     </row>
-    <row r="74" spans="1:9" ht="30" customHeight="1">
+    <row r="74" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B74" s="20">
         <v>3</v>
       </c>
@@ -1692,7 +1676,7 @@
       <c r="H74" s="8"/>
       <c r="I74" s="8"/>
     </row>
-    <row r="75" spans="1:9" ht="30" customHeight="1">
+    <row r="75" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B75" s="20">
         <v>4</v>
       </c>
@@ -1704,7 +1688,7 @@
       <c r="H75" s="8"/>
       <c r="I75" s="8"/>
     </row>
-    <row r="76" spans="1:9" ht="30" customHeight="1">
+    <row r="76" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B76" s="20">
         <v>5</v>
       </c>
@@ -1716,7 +1700,7 @@
       <c r="H76" s="8"/>
       <c r="I76" s="8"/>
     </row>
-    <row r="77" spans="1:9" ht="30" customHeight="1">
+    <row r="77" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B77" s="20">
         <v>6</v>
       </c>
@@ -1728,7 +1712,7 @@
       <c r="H77" s="8"/>
       <c r="I77" s="8"/>
     </row>
-    <row r="78" spans="1:9" ht="30" customHeight="1">
+    <row r="78" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B78" s="20">
         <v>7</v>
       </c>
@@ -1739,7 +1723,7 @@
       <c r="G78" s="5"/>
       <c r="H78" s="8"/>
     </row>
-    <row r="79" spans="1:9" ht="30" customHeight="1">
+    <row r="79" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B79" s="20">
         <v>8</v>
       </c>
@@ -1750,7 +1734,7 @@
       <c r="G79" s="5"/>
       <c r="H79" s="8"/>
     </row>
-    <row r="80" spans="1:9" ht="30" customHeight="1">
+    <row r="80" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B80" s="20">
         <v>9</v>
       </c>
@@ -1762,7 +1746,7 @@
       <c r="H80" s="8"/>
       <c r="I80" s="8"/>
     </row>
-    <row r="81" spans="1:9" ht="30" customHeight="1">
+    <row r="81" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B81" s="20">
         <v>10</v>
       </c>
@@ -1774,7 +1758,7 @@
       <c r="H81" s="8"/>
       <c r="I81" s="8"/>
     </row>
-    <row r="82" spans="1:9" ht="30" customHeight="1">
+    <row r="82" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B82" s="20">
         <v>11</v>
       </c>
@@ -1786,7 +1770,7 @@
       <c r="H82" s="8"/>
       <c r="I82" s="8"/>
     </row>
-    <row r="83" spans="1:9" ht="30" customHeight="1">
+    <row r="83" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B83" s="20">
         <v>12</v>
       </c>
@@ -1798,7 +1782,7 @@
       <c r="H83" s="8"/>
       <c r="I83" s="8"/>
     </row>
-    <row r="84" spans="1:9" ht="30" customHeight="1">
+    <row r="84" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B84" s="20">
         <v>13</v>
       </c>
@@ -1810,7 +1794,7 @@
       <c r="H84" s="8"/>
       <c r="I84" s="8"/>
     </row>
-    <row r="85" spans="1:9" ht="30" customHeight="1">
+    <row r="85" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B85" s="20">
         <v>14</v>
       </c>
@@ -1822,7 +1806,7 @@
       <c r="H85" s="8"/>
       <c r="I85" s="8"/>
     </row>
-    <row r="86" spans="1:9" ht="30" customHeight="1">
+    <row r="86" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B86" s="20">
         <v>15</v>
       </c>
@@ -1833,7 +1817,7 @@
       <c r="G86" s="5"/>
       <c r="H86" s="8"/>
     </row>
-    <row r="87" spans="1:9" ht="30" customHeight="1">
+    <row r="87" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B87" s="20">
         <v>16</v>
       </c>
@@ -1844,7 +1828,7 @@
       <c r="G87" s="5"/>
       <c r="H87" s="8"/>
     </row>
-    <row r="88" spans="1:9" ht="30" customHeight="1">
+    <row r="88" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B88" s="20">
         <v>17</v>
       </c>
@@ -1855,7 +1839,7 @@
       <c r="G88" s="5"/>
       <c r="H88" s="8"/>
     </row>
-    <row r="89" spans="1:9" ht="30" customHeight="1">
+    <row r="89" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B89" s="20">
         <v>18</v>
       </c>
@@ -1866,7 +1850,7 @@
       <c r="G89" s="5"/>
       <c r="H89" s="8"/>
     </row>
-    <row r="90" spans="1:9" ht="30" customHeight="1">
+    <row r="90" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B90" s="20">
         <v>19</v>
       </c>
@@ -1877,7 +1861,7 @@
       <c r="G90" s="5"/>
       <c r="H90" s="8"/>
     </row>
-    <row r="91" spans="1:9" ht="30" customHeight="1">
+    <row r="91" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B91" s="20">
         <v>20</v>
       </c>
@@ -1891,13 +1875,13 @@
       </c>
       <c r="H91" s="8"/>
     </row>
-    <row r="92" spans="1:9" ht="30" customHeight="1">
+    <row r="92" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B92" s="19"/>
       <c r="E92" s="12"/>
       <c r="F92" s="13"/>
       <c r="H92" s="8"/>
     </row>
-    <row r="93" spans="1:9" ht="30" customHeight="1">
+    <row r="93" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A93" s="15">
         <v>5</v>
       </c>
@@ -1908,7 +1892,7 @@
       <c r="F93" s="9"/>
       <c r="H93" s="8"/>
     </row>
-    <row r="94" spans="1:9" ht="30" customHeight="1">
+    <row r="94" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B94" s="20">
         <v>1</v>
       </c>
@@ -1919,7 +1903,7 @@
       <c r="G94" s="5"/>
       <c r="H94" s="8"/>
     </row>
-    <row r="95" spans="1:9" ht="30" customHeight="1">
+    <row r="95" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B95" s="20">
         <v>2</v>
       </c>
@@ -1930,7 +1914,7 @@
       <c r="G95" s="5"/>
       <c r="H95" s="8"/>
     </row>
-    <row r="96" spans="1:9" ht="30" customHeight="1">
+    <row r="96" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B96" s="20">
         <v>3</v>
       </c>
@@ -1941,7 +1925,7 @@
       <c r="G96" s="5"/>
       <c r="H96" s="8"/>
     </row>
-    <row r="97" spans="2:7" ht="30" customHeight="1">
+    <row r="97" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B97" s="20">
         <v>4</v>
       </c>
@@ -1951,7 +1935,7 @@
       <c r="F97" s="10"/>
       <c r="G97" s="5"/>
     </row>
-    <row r="98" spans="2:7" ht="30" customHeight="1">
+    <row r="98" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B98" s="20">
         <v>5</v>
       </c>
@@ -1961,7 +1945,7 @@
       <c r="F98" s="10"/>
       <c r="G98" s="5"/>
     </row>
-    <row r="99" spans="2:7" ht="30" customHeight="1">
+    <row r="99" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B99" s="20">
         <v>6</v>
       </c>
@@ -1971,7 +1955,7 @@
       <c r="F99" s="10"/>
       <c r="G99" s="5"/>
     </row>
-    <row r="100" spans="2:7" ht="30" customHeight="1">
+    <row r="100" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B100" s="20">
         <v>7</v>
       </c>
@@ -1981,7 +1965,7 @@
       <c r="F100" s="10"/>
       <c r="G100" s="5"/>
     </row>
-    <row r="101" spans="2:7" ht="30" customHeight="1">
+    <row r="101" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B101" s="20">
         <v>8</v>
       </c>
@@ -1991,7 +1975,7 @@
       <c r="F101" s="10"/>
       <c r="G101" s="5"/>
     </row>
-    <row r="102" spans="2:7" ht="30" customHeight="1">
+    <row r="102" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B102" s="20">
         <v>9</v>
       </c>
@@ -2001,7 +1985,7 @@
       <c r="F102" s="10"/>
       <c r="G102" s="5"/>
     </row>
-    <row r="103" spans="2:7" ht="30" customHeight="1">
+    <row r="103" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B103" s="20">
         <v>10</v>
       </c>
@@ -2011,7 +1995,7 @@
       <c r="F103" s="10"/>
       <c r="G103" s="5"/>
     </row>
-    <row r="104" spans="2:7" ht="30" customHeight="1">
+    <row r="104" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B104" s="20">
         <v>11</v>
       </c>
@@ -2021,7 +2005,7 @@
       <c r="F104" s="10"/>
       <c r="G104" s="5"/>
     </row>
-    <row r="105" spans="2:7" ht="30" customHeight="1">
+    <row r="105" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B105" s="20">
         <v>12</v>
       </c>
@@ -2031,7 +2015,7 @@
       <c r="F105" s="10"/>
       <c r="G105" s="5"/>
     </row>
-    <row r="106" spans="2:7" ht="30" customHeight="1">
+    <row r="106" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B106" s="20">
         <v>13</v>
       </c>
@@ -2041,7 +2025,7 @@
       <c r="F106" s="10"/>
       <c r="G106" s="5"/>
     </row>
-    <row r="107" spans="2:7" ht="30" customHeight="1">
+    <row r="107" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B107" s="20">
         <v>14</v>
       </c>
@@ -2051,7 +2035,7 @@
       <c r="F107" s="10"/>
       <c r="G107" s="5"/>
     </row>
-    <row r="108" spans="2:7" ht="30" customHeight="1">
+    <row r="108" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B108" s="20">
         <v>15</v>
       </c>
@@ -2061,7 +2045,7 @@
       <c r="F108" s="10"/>
       <c r="G108" s="5"/>
     </row>
-    <row r="109" spans="2:7" ht="30" customHeight="1">
+    <row r="109" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B109" s="20">
         <v>16</v>
       </c>
@@ -2071,7 +2055,7 @@
       <c r="F109" s="10"/>
       <c r="G109" s="5"/>
     </row>
-    <row r="110" spans="2:7" ht="30" customHeight="1">
+    <row r="110" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B110" s="20">
         <v>17</v>
       </c>
@@ -2081,7 +2065,7 @@
       <c r="F110" s="10"/>
       <c r="G110" s="5"/>
     </row>
-    <row r="111" spans="2:7" ht="30" customHeight="1">
+    <row r="111" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B111" s="20">
         <v>18</v>
       </c>
@@ -2091,7 +2075,7 @@
       <c r="F111" s="10"/>
       <c r="G111" s="5"/>
     </row>
-    <row r="112" spans="2:7" ht="30" customHeight="1">
+    <row r="112" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B112" s="20">
         <v>19</v>
       </c>
@@ -2101,7 +2085,7 @@
       <c r="F112" s="10"/>
       <c r="G112" s="5"/>
     </row>
-    <row r="113" spans="1:7" ht="30" customHeight="1">
+    <row r="113" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B113" s="20">
         <v>20</v>
       </c>
@@ -2114,12 +2098,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="114" spans="1:7" ht="30" customHeight="1">
+    <row r="114" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B114" s="19"/>
       <c r="E114" s="12"/>
       <c r="F114" s="13"/>
     </row>
-    <row r="115" spans="1:7" ht="30" customHeight="1">
+    <row r="115" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A115" s="15">
         <v>6</v>
       </c>
@@ -2129,7 +2113,7 @@
       </c>
       <c r="F115" s="9"/>
     </row>
-    <row r="116" spans="1:7" ht="30" customHeight="1">
+    <row r="116" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B116" s="20">
         <v>1</v>
       </c>
@@ -2139,7 +2123,7 @@
       <c r="F116" s="10"/>
       <c r="G116" s="5"/>
     </row>
-    <row r="117" spans="1:7" ht="30" customHeight="1">
+    <row r="117" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B117" s="20">
         <v>2</v>
       </c>
@@ -2149,7 +2133,7 @@
       <c r="F117" s="10"/>
       <c r="G117" s="5"/>
     </row>
-    <row r="118" spans="1:7" ht="30" customHeight="1">
+    <row r="118" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B118" s="20">
         <v>3</v>
       </c>
@@ -2159,7 +2143,7 @@
       <c r="F118" s="10"/>
       <c r="G118" s="5"/>
     </row>
-    <row r="119" spans="1:7" ht="30" customHeight="1">
+    <row r="119" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B119" s="20">
         <v>4</v>
       </c>
@@ -2169,7 +2153,7 @@
       <c r="F119" s="10"/>
       <c r="G119" s="5"/>
     </row>
-    <row r="120" spans="1:7" ht="30" customHeight="1">
+    <row r="120" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B120" s="20">
         <v>5</v>
       </c>
@@ -2179,7 +2163,7 @@
       <c r="F120" s="10"/>
       <c r="G120" s="5"/>
     </row>
-    <row r="121" spans="1:7" ht="30" customHeight="1">
+    <row r="121" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B121" s="20">
         <v>6</v>
       </c>
@@ -2189,7 +2173,7 @@
       <c r="F121" s="10"/>
       <c r="G121" s="5"/>
     </row>
-    <row r="122" spans="1:7" ht="30" customHeight="1">
+    <row r="122" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B122" s="20">
         <v>7</v>
       </c>
@@ -2199,7 +2183,7 @@
       <c r="F122" s="10"/>
       <c r="G122" s="5"/>
     </row>
-    <row r="123" spans="1:7" ht="30" customHeight="1">
+    <row r="123" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B123" s="20">
         <v>8</v>
       </c>
@@ -2209,7 +2193,7 @@
       <c r="F123" s="10"/>
       <c r="G123" s="5"/>
     </row>
-    <row r="124" spans="1:7" ht="30" customHeight="1">
+    <row r="124" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B124" s="20">
         <v>9</v>
       </c>
@@ -2219,7 +2203,7 @@
       <c r="F124" s="10"/>
       <c r="G124" s="5"/>
     </row>
-    <row r="125" spans="1:7" ht="30" customHeight="1">
+    <row r="125" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B125" s="20">
         <v>10</v>
       </c>
@@ -2229,7 +2213,7 @@
       <c r="F125" s="10"/>
       <c r="G125" s="5"/>
     </row>
-    <row r="126" spans="1:7" ht="30" customHeight="1">
+    <row r="126" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B126" s="20">
         <v>11</v>
       </c>
@@ -2239,7 +2223,7 @@
       <c r="F126" s="10"/>
       <c r="G126" s="5"/>
     </row>
-    <row r="127" spans="1:7" ht="30" customHeight="1">
+    <row r="127" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B127" s="20">
         <v>12</v>
       </c>
@@ -2249,7 +2233,7 @@
       <c r="F127" s="10"/>
       <c r="G127" s="5"/>
     </row>
-    <row r="128" spans="1:7" ht="30" customHeight="1">
+    <row r="128" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B128" s="20">
         <v>13</v>
       </c>
@@ -2259,7 +2243,7 @@
       <c r="F128" s="10"/>
       <c r="G128" s="5"/>
     </row>
-    <row r="129" spans="1:7" ht="30" customHeight="1">
+    <row r="129" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B129" s="20">
         <v>14</v>
       </c>
@@ -2269,7 +2253,7 @@
       <c r="F129" s="10"/>
       <c r="G129" s="5"/>
     </row>
-    <row r="130" spans="1:7" ht="30" customHeight="1">
+    <row r="130" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B130" s="20">
         <v>15</v>
       </c>
@@ -2279,7 +2263,7 @@
       <c r="F130" s="10"/>
       <c r="G130" s="5"/>
     </row>
-    <row r="131" spans="1:7" ht="30" customHeight="1">
+    <row r="131" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B131" s="20">
         <v>16</v>
       </c>
@@ -2289,7 +2273,7 @@
       <c r="F131" s="10"/>
       <c r="G131" s="5"/>
     </row>
-    <row r="132" spans="1:7" ht="30" customHeight="1">
+    <row r="132" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B132" s="20">
         <v>17</v>
       </c>
@@ -2299,7 +2283,7 @@
       <c r="F132" s="10"/>
       <c r="G132" s="5"/>
     </row>
-    <row r="133" spans="1:7" ht="30" customHeight="1">
+    <row r="133" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B133" s="20">
         <v>18</v>
       </c>
@@ -2309,7 +2293,7 @@
       <c r="F133" s="10"/>
       <c r="G133" s="5"/>
     </row>
-    <row r="134" spans="1:7" ht="30" customHeight="1">
+    <row r="134" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B134" s="20">
         <v>19</v>
       </c>
@@ -2319,7 +2303,7 @@
       <c r="F134" s="10"/>
       <c r="G134" s="5"/>
     </row>
-    <row r="135" spans="1:7" ht="30" customHeight="1">
+    <row r="135" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B135" s="20">
         <v>20</v>
       </c>
@@ -2332,12 +2316,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="136" spans="1:7" ht="30" customHeight="1">
+    <row r="136" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B136" s="19"/>
       <c r="E136" s="12"/>
       <c r="F136" s="13"/>
     </row>
-    <row r="137" spans="1:7" ht="30" customHeight="1">
+    <row r="137" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A137" s="15">
         <v>7</v>
       </c>
@@ -2347,7 +2331,7 @@
       </c>
       <c r="F137" s="9"/>
     </row>
-    <row r="138" spans="1:7" ht="30" customHeight="1">
+    <row r="138" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B138" s="20">
         <v>1</v>
       </c>
@@ -2357,7 +2341,7 @@
       <c r="F138" s="10"/>
       <c r="G138" s="5"/>
     </row>
-    <row r="139" spans="1:7" ht="30" customHeight="1">
+    <row r="139" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B139" s="20">
         <v>2</v>
       </c>
@@ -2367,7 +2351,7 @@
       <c r="F139" s="10"/>
       <c r="G139" s="5"/>
     </row>
-    <row r="140" spans="1:7" ht="30" customHeight="1">
+    <row r="140" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B140" s="20">
         <v>3</v>
       </c>
@@ -2377,7 +2361,7 @@
       <c r="F140" s="10"/>
       <c r="G140" s="5"/>
     </row>
-    <row r="141" spans="1:7" ht="30" customHeight="1">
+    <row r="141" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B141" s="20">
         <v>4</v>
       </c>
@@ -2387,7 +2371,7 @@
       <c r="F141" s="10"/>
       <c r="G141" s="5"/>
     </row>
-    <row r="142" spans="1:7" ht="30" customHeight="1">
+    <row r="142" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B142" s="20">
         <v>5</v>
       </c>
@@ -2397,7 +2381,7 @@
       <c r="F142" s="10"/>
       <c r="G142" s="5"/>
     </row>
-    <row r="143" spans="1:7" ht="30" customHeight="1">
+    <row r="143" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B143" s="20">
         <v>6</v>
       </c>
@@ -2407,7 +2391,7 @@
       <c r="F143" s="10"/>
       <c r="G143" s="5"/>
     </row>
-    <row r="144" spans="1:7" ht="30" customHeight="1">
+    <row r="144" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B144" s="20">
         <v>7</v>
       </c>
@@ -2417,7 +2401,7 @@
       <c r="F144" s="10"/>
       <c r="G144" s="5"/>
     </row>
-    <row r="145" spans="1:7" ht="30" customHeight="1">
+    <row r="145" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B145" s="20">
         <v>8</v>
       </c>
@@ -2427,7 +2411,7 @@
       <c r="F145" s="10"/>
       <c r="G145" s="5"/>
     </row>
-    <row r="146" spans="1:7" ht="30" customHeight="1">
+    <row r="146" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B146" s="20">
         <v>9</v>
       </c>
@@ -2437,7 +2421,7 @@
       <c r="F146" s="10"/>
       <c r="G146" s="5"/>
     </row>
-    <row r="147" spans="1:7" ht="30" customHeight="1">
+    <row r="147" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B147" s="20">
         <v>10</v>
       </c>
@@ -2447,7 +2431,7 @@
       <c r="F147" s="10"/>
       <c r="G147" s="5"/>
     </row>
-    <row r="148" spans="1:7" ht="30" customHeight="1">
+    <row r="148" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B148" s="20">
         <v>11</v>
       </c>
@@ -2457,7 +2441,7 @@
       <c r="F148" s="10"/>
       <c r="G148" s="5"/>
     </row>
-    <row r="149" spans="1:7" ht="30" customHeight="1">
+    <row r="149" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B149" s="20">
         <v>12</v>
       </c>
@@ -2467,7 +2451,7 @@
       <c r="F149" s="10"/>
       <c r="G149" s="5"/>
     </row>
-    <row r="150" spans="1:7" ht="30" customHeight="1">
+    <row r="150" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B150" s="20">
         <v>13</v>
       </c>
@@ -2477,7 +2461,7 @@
       <c r="F150" s="10"/>
       <c r="G150" s="5"/>
     </row>
-    <row r="151" spans="1:7" ht="30" customHeight="1">
+    <row r="151" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B151" s="20">
         <v>14</v>
       </c>
@@ -2487,7 +2471,7 @@
       <c r="F151" s="10"/>
       <c r="G151" s="5"/>
     </row>
-    <row r="152" spans="1:7" ht="30" customHeight="1">
+    <row r="152" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B152" s="20">
         <v>15</v>
       </c>
@@ -2497,7 +2481,7 @@
       <c r="F152" s="10"/>
       <c r="G152" s="5"/>
     </row>
-    <row r="153" spans="1:7" ht="30" customHeight="1">
+    <row r="153" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B153" s="20">
         <v>16</v>
       </c>
@@ -2507,7 +2491,7 @@
       <c r="F153" s="10"/>
       <c r="G153" s="5"/>
     </row>
-    <row r="154" spans="1:7" ht="30" customHeight="1">
+    <row r="154" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B154" s="20">
         <v>17</v>
       </c>
@@ -2517,7 +2501,7 @@
       <c r="F154" s="10"/>
       <c r="G154" s="5"/>
     </row>
-    <row r="155" spans="1:7" ht="30" customHeight="1">
+    <row r="155" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B155" s="20">
         <v>18</v>
       </c>
@@ -2527,7 +2511,7 @@
       <c r="F155" s="10"/>
       <c r="G155" s="5"/>
     </row>
-    <row r="156" spans="1:7" ht="30" customHeight="1">
+    <row r="156" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B156" s="20">
         <v>19</v>
       </c>
@@ -2537,7 +2521,7 @@
       <c r="F156" s="10"/>
       <c r="G156" s="5"/>
     </row>
-    <row r="157" spans="1:7" ht="30" customHeight="1">
+    <row r="157" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B157" s="20">
         <v>20</v>
       </c>
@@ -2550,12 +2534,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="158" spans="1:7" ht="30" customHeight="1">
+    <row r="158" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B158" s="19"/>
       <c r="E158" s="12"/>
       <c r="F158" s="13"/>
     </row>
-    <row r="159" spans="1:7" ht="30" customHeight="1">
+    <row r="159" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A159" s="15">
         <v>8</v>
       </c>
@@ -2565,7 +2549,7 @@
       </c>
       <c r="F159" s="9"/>
     </row>
-    <row r="160" spans="1:7" ht="30" customHeight="1">
+    <row r="160" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B160" s="20">
         <v>1</v>
       </c>
@@ -2575,7 +2559,7 @@
       <c r="F160" s="10"/>
       <c r="G160" s="5"/>
     </row>
-    <row r="161" spans="2:7" ht="30" customHeight="1">
+    <row r="161" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B161" s="20">
         <v>2</v>
       </c>
@@ -2585,7 +2569,7 @@
       <c r="F161" s="10"/>
       <c r="G161" s="5"/>
     </row>
-    <row r="162" spans="2:7" ht="30" customHeight="1">
+    <row r="162" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B162" s="20">
         <v>3</v>
       </c>
@@ -2595,7 +2579,7 @@
       <c r="F162" s="10"/>
       <c r="G162" s="5"/>
     </row>
-    <row r="163" spans="2:7" ht="30" customHeight="1">
+    <row r="163" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B163" s="20">
         <v>4</v>
       </c>
@@ -2605,7 +2589,7 @@
       <c r="F163" s="10"/>
       <c r="G163" s="5"/>
     </row>
-    <row r="164" spans="2:7" ht="30" customHeight="1">
+    <row r="164" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B164" s="20">
         <v>5</v>
       </c>
@@ -2615,7 +2599,7 @@
       <c r="F164" s="10"/>
       <c r="G164" s="5"/>
     </row>
-    <row r="165" spans="2:7" ht="30" customHeight="1">
+    <row r="165" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B165" s="20">
         <v>6</v>
       </c>
@@ -2625,7 +2609,7 @@
       <c r="F165" s="10"/>
       <c r="G165" s="5"/>
     </row>
-    <row r="166" spans="2:7" ht="30" customHeight="1">
+    <row r="166" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B166" s="20">
         <v>7</v>
       </c>
@@ -2635,7 +2619,7 @@
       <c r="F166" s="10"/>
       <c r="G166" s="5"/>
     </row>
-    <row r="167" spans="2:7" ht="30" customHeight="1">
+    <row r="167" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B167" s="20">
         <v>8</v>
       </c>
@@ -2645,7 +2629,7 @@
       <c r="F167" s="10"/>
       <c r="G167" s="5"/>
     </row>
-    <row r="168" spans="2:7" ht="30" customHeight="1">
+    <row r="168" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B168" s="20">
         <v>9</v>
       </c>
@@ -2655,7 +2639,7 @@
       <c r="F168" s="10"/>
       <c r="G168" s="5"/>
     </row>
-    <row r="169" spans="2:7" ht="30" customHeight="1">
+    <row r="169" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B169" s="20">
         <v>10</v>
       </c>
@@ -2665,7 +2649,7 @@
       <c r="F169" s="10"/>
       <c r="G169" s="5"/>
     </row>
-    <row r="170" spans="2:7" ht="30" customHeight="1">
+    <row r="170" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B170" s="20">
         <v>11</v>
       </c>
@@ -2675,7 +2659,7 @@
       <c r="F170" s="10"/>
       <c r="G170" s="5"/>
     </row>
-    <row r="171" spans="2:7" ht="30" customHeight="1">
+    <row r="171" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B171" s="20">
         <v>12</v>
       </c>
@@ -2685,7 +2669,7 @@
       <c r="F171" s="10"/>
       <c r="G171" s="5"/>
     </row>
-    <row r="172" spans="2:7" ht="30" customHeight="1">
+    <row r="172" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B172" s="20">
         <v>13</v>
       </c>
@@ -2695,7 +2679,7 @@
       <c r="F172" s="10"/>
       <c r="G172" s="5"/>
     </row>
-    <row r="173" spans="2:7" ht="30" customHeight="1">
+    <row r="173" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B173" s="20">
         <v>14</v>
       </c>
@@ -2705,7 +2689,7 @@
       <c r="F173" s="10"/>
       <c r="G173" s="5"/>
     </row>
-    <row r="174" spans="2:7" ht="30" customHeight="1">
+    <row r="174" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B174" s="20">
         <v>15</v>
       </c>
@@ -2715,7 +2699,7 @@
       <c r="F174" s="10"/>
       <c r="G174" s="5"/>
     </row>
-    <row r="175" spans="2:7" ht="30" customHeight="1">
+    <row r="175" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B175" s="20">
         <v>16</v>
       </c>
@@ -2725,7 +2709,7 @@
       <c r="F175" s="10"/>
       <c r="G175" s="5"/>
     </row>
-    <row r="176" spans="2:7" ht="30" customHeight="1">
+    <row r="176" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B176" s="20">
         <v>17</v>
       </c>
@@ -2735,7 +2719,7 @@
       <c r="F176" s="10"/>
       <c r="G176" s="5"/>
     </row>
-    <row r="177" spans="1:7" ht="30" customHeight="1">
+    <row r="177" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B177" s="20">
         <v>18</v>
       </c>
@@ -2745,7 +2729,7 @@
       <c r="F177" s="10"/>
       <c r="G177" s="5"/>
     </row>
-    <row r="178" spans="1:7" ht="30" customHeight="1">
+    <row r="178" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B178" s="20">
         <v>19</v>
       </c>
@@ -2755,7 +2739,7 @@
       <c r="F178" s="10"/>
       <c r="G178" s="5"/>
     </row>
-    <row r="179" spans="1:7" ht="30" customHeight="1">
+    <row r="179" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B179" s="20">
         <v>20</v>
       </c>
@@ -2768,12 +2752,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="180" spans="1:7" ht="30" customHeight="1">
+    <row r="180" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B180" s="19"/>
       <c r="E180" s="12"/>
       <c r="F180" s="13"/>
     </row>
-    <row r="181" spans="1:7" ht="30" customHeight="1">
+    <row r="181" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A181" s="15">
         <v>9</v>
       </c>
@@ -2783,7 +2767,7 @@
       </c>
       <c r="F181" s="9"/>
     </row>
-    <row r="182" spans="1:7" ht="30" customHeight="1">
+    <row r="182" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B182" s="20">
         <v>1</v>
       </c>
@@ -2793,7 +2777,7 @@
       <c r="F182" s="10"/>
       <c r="G182" s="5"/>
     </row>
-    <row r="183" spans="1:7" ht="30" customHeight="1">
+    <row r="183" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B183" s="20">
         <v>2</v>
       </c>
@@ -2803,7 +2787,7 @@
       <c r="F183" s="10"/>
       <c r="G183" s="5"/>
     </row>
-    <row r="184" spans="1:7" ht="30" customHeight="1">
+    <row r="184" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B184" s="20">
         <v>3</v>
       </c>
@@ -2813,7 +2797,7 @@
       <c r="F184" s="10"/>
       <c r="G184" s="5"/>
     </row>
-    <row r="185" spans="1:7" ht="30" customHeight="1">
+    <row r="185" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B185" s="20">
         <v>4</v>
       </c>
@@ -2823,7 +2807,7 @@
       <c r="F185" s="10"/>
       <c r="G185" s="5"/>
     </row>
-    <row r="186" spans="1:7" ht="30" customHeight="1">
+    <row r="186" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B186" s="20">
         <v>5</v>
       </c>
@@ -2833,7 +2817,7 @@
       <c r="F186" s="10"/>
       <c r="G186" s="5"/>
     </row>
-    <row r="187" spans="1:7" ht="30" customHeight="1">
+    <row r="187" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B187" s="20">
         <v>6</v>
       </c>
@@ -2843,7 +2827,7 @@
       <c r="F187" s="10"/>
       <c r="G187" s="5"/>
     </row>
-    <row r="188" spans="1:7" ht="30" customHeight="1">
+    <row r="188" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B188" s="20">
         <v>7</v>
       </c>
@@ -2853,7 +2837,7 @@
       <c r="F188" s="10"/>
       <c r="G188" s="5"/>
     </row>
-    <row r="189" spans="1:7" ht="30" customHeight="1">
+    <row r="189" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B189" s="20">
         <v>8</v>
       </c>
@@ -2863,7 +2847,7 @@
       <c r="F189" s="10"/>
       <c r="G189" s="5"/>
     </row>
-    <row r="190" spans="1:7" ht="30" customHeight="1">
+    <row r="190" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B190" s="20">
         <v>9</v>
       </c>
@@ -2873,7 +2857,7 @@
       <c r="F190" s="10"/>
       <c r="G190" s="5"/>
     </row>
-    <row r="191" spans="1:7" ht="30" customHeight="1">
+    <row r="191" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B191" s="20">
         <v>10</v>
       </c>
@@ -2883,7 +2867,7 @@
       <c r="F191" s="10"/>
       <c r="G191" s="5"/>
     </row>
-    <row r="192" spans="1:7" ht="30" customHeight="1">
+    <row r="192" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B192" s="20">
         <v>11</v>
       </c>
@@ -2893,7 +2877,7 @@
       <c r="F192" s="10"/>
       <c r="G192" s="5"/>
     </row>
-    <row r="193" spans="1:7" ht="30" customHeight="1">
+    <row r="193" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B193" s="20">
         <v>12</v>
       </c>
@@ -2903,7 +2887,7 @@
       <c r="F193" s="10"/>
       <c r="G193" s="5"/>
     </row>
-    <row r="194" spans="1:7" ht="30" customHeight="1">
+    <row r="194" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B194" s="20">
         <v>13</v>
       </c>
@@ -2913,7 +2897,7 @@
       <c r="F194" s="10"/>
       <c r="G194" s="5"/>
     </row>
-    <row r="195" spans="1:7" ht="30" customHeight="1">
+    <row r="195" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B195" s="20">
         <v>14</v>
       </c>
@@ -2923,7 +2907,7 @@
       <c r="F195" s="10"/>
       <c r="G195" s="5"/>
     </row>
-    <row r="196" spans="1:7" ht="30" customHeight="1">
+    <row r="196" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B196" s="20">
         <v>15</v>
       </c>
@@ -2933,7 +2917,7 @@
       <c r="F196" s="10"/>
       <c r="G196" s="5"/>
     </row>
-    <row r="197" spans="1:7" ht="30" customHeight="1">
+    <row r="197" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B197" s="20">
         <v>16</v>
       </c>
@@ -2943,7 +2927,7 @@
       <c r="F197" s="10"/>
       <c r="G197" s="5"/>
     </row>
-    <row r="198" spans="1:7" ht="30" customHeight="1">
+    <row r="198" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B198" s="20">
         <v>17</v>
       </c>
@@ -2953,7 +2937,7 @@
       <c r="F198" s="10"/>
       <c r="G198" s="5"/>
     </row>
-    <row r="199" spans="1:7" ht="30" customHeight="1">
+    <row r="199" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B199" s="20">
         <v>18</v>
       </c>
@@ -2963,7 +2947,7 @@
       <c r="F199" s="10"/>
       <c r="G199" s="5"/>
     </row>
-    <row r="200" spans="1:7" ht="30" customHeight="1">
+    <row r="200" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B200" s="20">
         <v>19</v>
       </c>
@@ -2973,7 +2957,7 @@
       <c r="F200" s="10"/>
       <c r="G200" s="5"/>
     </row>
-    <row r="201" spans="1:7" ht="30" customHeight="1">
+    <row r="201" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B201" s="20">
         <v>20</v>
       </c>
@@ -2986,12 +2970,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="202" spans="1:7" ht="30" customHeight="1">
+    <row r="202" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B202" s="19"/>
       <c r="E202" s="12"/>
       <c r="F202" s="13"/>
     </row>
-    <row r="203" spans="1:7" ht="30" customHeight="1">
+    <row r="203" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A203" s="15">
         <v>10</v>
       </c>
@@ -3001,7 +2985,7 @@
       </c>
       <c r="F203" s="9"/>
     </row>
-    <row r="204" spans="1:7" ht="30" customHeight="1">
+    <row r="204" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B204" s="20">
         <v>1</v>
       </c>
@@ -3011,7 +2995,7 @@
       <c r="F204" s="10"/>
       <c r="G204" s="5"/>
     </row>
-    <row r="205" spans="1:7" ht="30" customHeight="1">
+    <row r="205" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B205" s="20">
         <v>2</v>
       </c>
@@ -3021,7 +3005,7 @@
       <c r="F205" s="10"/>
       <c r="G205" s="5"/>
     </row>
-    <row r="206" spans="1:7" ht="30" customHeight="1">
+    <row r="206" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B206" s="20">
         <v>3</v>
       </c>
@@ -3031,7 +3015,7 @@
       <c r="F206" s="10"/>
       <c r="G206" s="5"/>
     </row>
-    <row r="207" spans="1:7" ht="30" customHeight="1">
+    <row r="207" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B207" s="20">
         <v>4</v>
       </c>
@@ -3041,7 +3025,7 @@
       <c r="F207" s="10"/>
       <c r="G207" s="5"/>
     </row>
-    <row r="208" spans="1:7" ht="30" customHeight="1">
+    <row r="208" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B208" s="20">
         <v>5</v>
       </c>
@@ -3051,7 +3035,7 @@
       <c r="F208" s="10"/>
       <c r="G208" s="5"/>
     </row>
-    <row r="209" spans="2:7" ht="30" customHeight="1">
+    <row r="209" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B209" s="20">
         <v>6</v>
       </c>
@@ -3061,7 +3045,7 @@
       <c r="F209" s="10"/>
       <c r="G209" s="5"/>
     </row>
-    <row r="210" spans="2:7" ht="30" customHeight="1">
+    <row r="210" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B210" s="20">
         <v>7</v>
       </c>
@@ -3071,7 +3055,7 @@
       <c r="F210" s="10"/>
       <c r="G210" s="5"/>
     </row>
-    <row r="211" spans="2:7" ht="30" customHeight="1">
+    <row r="211" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B211" s="20">
         <v>8</v>
       </c>
@@ -3081,7 +3065,7 @@
       <c r="F211" s="10"/>
       <c r="G211" s="5"/>
     </row>
-    <row r="212" spans="2:7" ht="30" customHeight="1">
+    <row r="212" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B212" s="20">
         <v>9</v>
       </c>
@@ -3091,7 +3075,7 @@
       <c r="F212" s="10"/>
       <c r="G212" s="5"/>
     </row>
-    <row r="213" spans="2:7" ht="30" customHeight="1">
+    <row r="213" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B213" s="20">
         <v>10</v>
       </c>
@@ -3101,7 +3085,7 @@
       <c r="F213" s="10"/>
       <c r="G213" s="5"/>
     </row>
-    <row r="214" spans="2:7" ht="30" customHeight="1">
+    <row r="214" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B214" s="20">
         <v>11</v>
       </c>
@@ -3111,7 +3095,7 @@
       <c r="F214" s="10"/>
       <c r="G214" s="5"/>
     </row>
-    <row r="215" spans="2:7" ht="30" customHeight="1">
+    <row r="215" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B215" s="20">
         <v>12</v>
       </c>
@@ -3121,7 +3105,7 @@
       <c r="F215" s="10"/>
       <c r="G215" s="5"/>
     </row>
-    <row r="216" spans="2:7" ht="30" customHeight="1">
+    <row r="216" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B216" s="20">
         <v>13</v>
       </c>
@@ -3131,7 +3115,7 @@
       <c r="F216" s="10"/>
       <c r="G216" s="5"/>
     </row>
-    <row r="217" spans="2:7" ht="30" customHeight="1">
+    <row r="217" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B217" s="20">
         <v>14</v>
       </c>
@@ -3141,7 +3125,7 @@
       <c r="F217" s="10"/>
       <c r="G217" s="5"/>
     </row>
-    <row r="218" spans="2:7" ht="30" customHeight="1">
+    <row r="218" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B218" s="20">
         <v>15</v>
       </c>
@@ -3151,7 +3135,7 @@
       <c r="F218" s="10"/>
       <c r="G218" s="5"/>
     </row>
-    <row r="219" spans="2:7" ht="30" customHeight="1">
+    <row r="219" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B219" s="20">
         <v>16</v>
       </c>
@@ -3161,7 +3145,7 @@
       <c r="F219" s="10"/>
       <c r="G219" s="5"/>
     </row>
-    <row r="220" spans="2:7" ht="30" customHeight="1">
+    <row r="220" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B220" s="20">
         <v>17</v>
       </c>
@@ -3171,7 +3155,7 @@
       <c r="F220" s="10"/>
       <c r="G220" s="5"/>
     </row>
-    <row r="221" spans="2:7" ht="30" customHeight="1">
+    <row r="221" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B221" s="20">
         <v>18</v>
       </c>
@@ -3181,7 +3165,7 @@
       <c r="F221" s="10"/>
       <c r="G221" s="5"/>
     </row>
-    <row r="222" spans="2:7" ht="30" customHeight="1">
+    <row r="222" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B222" s="20">
         <v>19</v>
       </c>
@@ -3191,7 +3175,7 @@
       <c r="F222" s="10"/>
       <c r="G222" s="5"/>
     </row>
-    <row r="223" spans="2:7" ht="30" customHeight="1">
+    <row r="223" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B223" s="20">
         <v>20</v>
       </c>
@@ -3204,12 +3188,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="224" spans="2:7" ht="30" customHeight="1">
+    <row r="224" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B224" s="19"/>
       <c r="E224" s="12"/>
       <c r="F224" s="13"/>
     </row>
-    <row r="225" spans="1:7" ht="30" customHeight="1">
+    <row r="225" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A225" s="15">
         <v>11</v>
       </c>
@@ -3219,7 +3203,7 @@
       </c>
       <c r="F225" s="9"/>
     </row>
-    <row r="226" spans="1:7" ht="30" customHeight="1">
+    <row r="226" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B226" s="20">
         <v>1</v>
       </c>
@@ -3229,7 +3213,7 @@
       <c r="F226" s="10"/>
       <c r="G226" s="5"/>
     </row>
-    <row r="227" spans="1:7" ht="30" customHeight="1">
+    <row r="227" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B227" s="20">
         <v>2</v>
       </c>
@@ -3239,7 +3223,7 @@
       <c r="F227" s="10"/>
       <c r="G227" s="5"/>
     </row>
-    <row r="228" spans="1:7" ht="30" customHeight="1">
+    <row r="228" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B228" s="20">
         <v>3</v>
       </c>
@@ -3249,7 +3233,7 @@
       <c r="F228" s="10"/>
       <c r="G228" s="5"/>
     </row>
-    <row r="229" spans="1:7" ht="30" customHeight="1">
+    <row r="229" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B229" s="20">
         <v>4</v>
       </c>
@@ -3259,7 +3243,7 @@
       <c r="F229" s="10"/>
       <c r="G229" s="5"/>
     </row>
-    <row r="230" spans="1:7" ht="30" customHeight="1">
+    <row r="230" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B230" s="20">
         <v>5</v>
       </c>
@@ -3269,7 +3253,7 @@
       <c r="F230" s="10"/>
       <c r="G230" s="5"/>
     </row>
-    <row r="231" spans="1:7" ht="30" customHeight="1">
+    <row r="231" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B231" s="20">
         <v>6</v>
       </c>
@@ -3279,7 +3263,7 @@
       <c r="F231" s="10"/>
       <c r="G231" s="5"/>
     </row>
-    <row r="232" spans="1:7" ht="30" customHeight="1">
+    <row r="232" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B232" s="20">
         <v>7</v>
       </c>
@@ -3289,7 +3273,7 @@
       <c r="F232" s="10"/>
       <c r="G232" s="5"/>
     </row>
-    <row r="233" spans="1:7" ht="30" customHeight="1">
+    <row r="233" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B233" s="20">
         <v>8</v>
       </c>
@@ -3299,7 +3283,7 @@
       <c r="F233" s="10"/>
       <c r="G233" s="5"/>
     </row>
-    <row r="234" spans="1:7" ht="30" customHeight="1">
+    <row r="234" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B234" s="20">
         <v>9</v>
       </c>
@@ -3309,7 +3293,7 @@
       <c r="F234" s="10"/>
       <c r="G234" s="5"/>
     </row>
-    <row r="235" spans="1:7" ht="30" customHeight="1">
+    <row r="235" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B235" s="20">
         <v>10</v>
       </c>
@@ -3319,7 +3303,7 @@
       <c r="F235" s="10"/>
       <c r="G235" s="5"/>
     </row>
-    <row r="236" spans="1:7" ht="30" customHeight="1">
+    <row r="236" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B236" s="20">
         <v>11</v>
       </c>
@@ -3329,7 +3313,7 @@
       <c r="F236" s="10"/>
       <c r="G236" s="5"/>
     </row>
-    <row r="237" spans="1:7" ht="30" customHeight="1">
+    <row r="237" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B237" s="20">
         <v>12</v>
       </c>
@@ -3339,7 +3323,7 @@
       <c r="F237" s="10"/>
       <c r="G237" s="5"/>
     </row>
-    <row r="238" spans="1:7" ht="30" customHeight="1">
+    <row r="238" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B238" s="20">
         <v>13</v>
       </c>
@@ -3349,7 +3333,7 @@
       <c r="F238" s="10"/>
       <c r="G238" s="5"/>
     </row>
-    <row r="239" spans="1:7" ht="30" customHeight="1">
+    <row r="239" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B239" s="20">
         <v>14</v>
       </c>
@@ -3359,7 +3343,7 @@
       <c r="F239" s="10"/>
       <c r="G239" s="5"/>
     </row>
-    <row r="240" spans="1:7" ht="30" customHeight="1">
+    <row r="240" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B240" s="20">
         <v>15</v>
       </c>
@@ -3369,7 +3353,7 @@
       <c r="F240" s="10"/>
       <c r="G240" s="5"/>
     </row>
-    <row r="241" spans="1:7" ht="30" customHeight="1">
+    <row r="241" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B241" s="20">
         <v>16</v>
       </c>
@@ -3379,7 +3363,7 @@
       <c r="F241" s="10"/>
       <c r="G241" s="5"/>
     </row>
-    <row r="242" spans="1:7" ht="30" customHeight="1">
+    <row r="242" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B242" s="20">
         <v>17</v>
       </c>
@@ -3389,7 +3373,7 @@
       <c r="F242" s="10"/>
       <c r="G242" s="5"/>
     </row>
-    <row r="243" spans="1:7" ht="30" customHeight="1">
+    <row r="243" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B243" s="20">
         <v>18</v>
       </c>
@@ -3399,7 +3383,7 @@
       <c r="F243" s="10"/>
       <c r="G243" s="5"/>
     </row>
-    <row r="244" spans="1:7" ht="30" customHeight="1">
+    <row r="244" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B244" s="20">
         <v>19</v>
       </c>
@@ -3409,7 +3393,7 @@
       <c r="F244" s="10"/>
       <c r="G244" s="5"/>
     </row>
-    <row r="245" spans="1:7" ht="30" customHeight="1">
+    <row r="245" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B245" s="20">
         <v>20</v>
       </c>
@@ -3422,12 +3406,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="246" spans="1:7" ht="30" customHeight="1">
+    <row r="246" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B246" s="19"/>
       <c r="E246" s="12"/>
       <c r="F246" s="13"/>
     </row>
-    <row r="247" spans="1:7" ht="30" customHeight="1">
+    <row r="247" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A247" s="15">
         <v>12</v>
       </c>
@@ -3437,7 +3421,7 @@
       </c>
       <c r="F247" s="9"/>
     </row>
-    <row r="248" spans="1:7" ht="30" customHeight="1">
+    <row r="248" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B248" s="20">
         <v>1</v>
       </c>
@@ -3447,7 +3431,7 @@
       <c r="F248" s="10"/>
       <c r="G248" s="5"/>
     </row>
-    <row r="249" spans="1:7" ht="30" customHeight="1">
+    <row r="249" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B249" s="20">
         <v>2</v>
       </c>
@@ -3457,7 +3441,7 @@
       <c r="F249" s="10"/>
       <c r="G249" s="5"/>
     </row>
-    <row r="250" spans="1:7" ht="30" customHeight="1">
+    <row r="250" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B250" s="20">
         <v>3</v>
       </c>
@@ -3467,7 +3451,7 @@
       <c r="F250" s="10"/>
       <c r="G250" s="5"/>
     </row>
-    <row r="251" spans="1:7" ht="30" customHeight="1">
+    <row r="251" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B251" s="20">
         <v>4</v>
       </c>
@@ -3477,7 +3461,7 @@
       <c r="F251" s="10"/>
       <c r="G251" s="5"/>
     </row>
-    <row r="252" spans="1:7" ht="30" customHeight="1">
+    <row r="252" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B252" s="20">
         <v>5</v>
       </c>
@@ -3487,7 +3471,7 @@
       <c r="F252" s="10"/>
       <c r="G252" s="5"/>
     </row>
-    <row r="253" spans="1:7" ht="30" customHeight="1">
+    <row r="253" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B253" s="20">
         <v>6</v>
       </c>
@@ -3497,7 +3481,7 @@
       <c r="F253" s="10"/>
       <c r="G253" s="5"/>
     </row>
-    <row r="254" spans="1:7" ht="30" customHeight="1">
+    <row r="254" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B254" s="20">
         <v>7</v>
       </c>
@@ -3507,7 +3491,7 @@
       <c r="F254" s="10"/>
       <c r="G254" s="5"/>
     </row>
-    <row r="255" spans="1:7" ht="30" customHeight="1">
+    <row r="255" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B255" s="20">
         <v>8</v>
       </c>
@@ -3517,7 +3501,7 @@
       <c r="F255" s="10"/>
       <c r="G255" s="5"/>
     </row>
-    <row r="256" spans="1:7" ht="30" customHeight="1">
+    <row r="256" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B256" s="20">
         <v>9</v>
       </c>
@@ -3527,7 +3511,7 @@
       <c r="F256" s="10"/>
       <c r="G256" s="5"/>
     </row>
-    <row r="257" spans="1:7" ht="30" customHeight="1">
+    <row r="257" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B257" s="20">
         <v>10</v>
       </c>
@@ -3537,7 +3521,7 @@
       <c r="F257" s="10"/>
       <c r="G257" s="5"/>
     </row>
-    <row r="258" spans="1:7" ht="30" customHeight="1">
+    <row r="258" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B258" s="20">
         <v>11</v>
       </c>
@@ -3547,7 +3531,7 @@
       <c r="F258" s="10"/>
       <c r="G258" s="5"/>
     </row>
-    <row r="259" spans="1:7" ht="30" customHeight="1">
+    <row r="259" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B259" s="20">
         <v>12</v>
       </c>
@@ -3557,7 +3541,7 @@
       <c r="F259" s="10"/>
       <c r="G259" s="5"/>
     </row>
-    <row r="260" spans="1:7" ht="30" customHeight="1">
+    <row r="260" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B260" s="20">
         <v>13</v>
       </c>
@@ -3567,7 +3551,7 @@
       <c r="F260" s="10"/>
       <c r="G260" s="5"/>
     </row>
-    <row r="261" spans="1:7" ht="30" customHeight="1">
+    <row r="261" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B261" s="20">
         <v>14</v>
       </c>
@@ -3577,7 +3561,7 @@
       <c r="F261" s="10"/>
       <c r="G261" s="5"/>
     </row>
-    <row r="262" spans="1:7" ht="30" customHeight="1">
+    <row r="262" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B262" s="20">
         <v>15</v>
       </c>
@@ -3587,7 +3571,7 @@
       <c r="F262" s="10"/>
       <c r="G262" s="5"/>
     </row>
-    <row r="263" spans="1:7" ht="30" customHeight="1">
+    <row r="263" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B263" s="20">
         <v>16</v>
       </c>
@@ -3597,7 +3581,7 @@
       <c r="F263" s="10"/>
       <c r="G263" s="5"/>
     </row>
-    <row r="264" spans="1:7" ht="30" customHeight="1">
+    <row r="264" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B264" s="20">
         <v>17</v>
       </c>
@@ -3607,7 +3591,7 @@
       <c r="F264" s="10"/>
       <c r="G264" s="5"/>
     </row>
-    <row r="265" spans="1:7" ht="30" customHeight="1">
+    <row r="265" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B265" s="20">
         <v>18</v>
       </c>
@@ -3617,7 +3601,7 @@
       <c r="F265" s="10"/>
       <c r="G265" s="5"/>
     </row>
-    <row r="266" spans="1:7" ht="30" customHeight="1">
+    <row r="266" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B266" s="20">
         <v>19</v>
       </c>
@@ -3627,7 +3611,7 @@
       <c r="F266" s="10"/>
       <c r="G266" s="5"/>
     </row>
-    <row r="267" spans="1:7" ht="30" customHeight="1">
+    <row r="267" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B267" s="20">
         <v>20</v>
       </c>
@@ -3640,12 +3624,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="268" spans="1:7" ht="30" customHeight="1">
+    <row r="268" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B268" s="19"/>
       <c r="E268" s="12"/>
       <c r="F268" s="13"/>
     </row>
-    <row r="269" spans="1:7" ht="30" customHeight="1">
+    <row r="269" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A269" s="15">
         <v>13</v>
       </c>
@@ -3655,7 +3639,7 @@
       </c>
       <c r="F269" s="9"/>
     </row>
-    <row r="270" spans="1:7" ht="30" customHeight="1">
+    <row r="270" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B270" s="20">
         <v>1</v>
       </c>
@@ -3665,7 +3649,7 @@
       <c r="F270" s="10"/>
       <c r="G270" s="5"/>
     </row>
-    <row r="271" spans="1:7" ht="30" customHeight="1">
+    <row r="271" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B271" s="20">
         <v>2</v>
       </c>
@@ -3675,7 +3659,7 @@
       <c r="F271" s="10"/>
       <c r="G271" s="5"/>
     </row>
-    <row r="272" spans="1:7" ht="30" customHeight="1">
+    <row r="272" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B272" s="20">
         <v>3</v>
       </c>
@@ -3685,7 +3669,7 @@
       <c r="F272" s="10"/>
       <c r="G272" s="5"/>
     </row>
-    <row r="273" spans="2:7" ht="30" customHeight="1">
+    <row r="273" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B273" s="20">
         <v>4</v>
       </c>
@@ -3695,7 +3679,7 @@
       <c r="F273" s="10"/>
       <c r="G273" s="5"/>
     </row>
-    <row r="274" spans="2:7" ht="30" customHeight="1">
+    <row r="274" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B274" s="20">
         <v>5</v>
       </c>
@@ -3705,7 +3689,7 @@
       <c r="F274" s="10"/>
       <c r="G274" s="5"/>
     </row>
-    <row r="275" spans="2:7" ht="30" customHeight="1">
+    <row r="275" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B275" s="20">
         <v>6</v>
       </c>
@@ -3715,7 +3699,7 @@
       <c r="F275" s="10"/>
       <c r="G275" s="5"/>
     </row>
-    <row r="276" spans="2:7" ht="30" customHeight="1">
+    <row r="276" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B276" s="20">
         <v>7</v>
       </c>
@@ -3725,7 +3709,7 @@
       <c r="F276" s="10"/>
       <c r="G276" s="5"/>
     </row>
-    <row r="277" spans="2:7" ht="30" customHeight="1">
+    <row r="277" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B277" s="20">
         <v>8</v>
       </c>
@@ -3735,7 +3719,7 @@
       <c r="F277" s="10"/>
       <c r="G277" s="5"/>
     </row>
-    <row r="278" spans="2:7" ht="30" customHeight="1">
+    <row r="278" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B278" s="20">
         <v>9</v>
       </c>
@@ -3745,7 +3729,7 @@
       <c r="F278" s="10"/>
       <c r="G278" s="5"/>
     </row>
-    <row r="279" spans="2:7" ht="30" customHeight="1">
+    <row r="279" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B279" s="20">
         <v>10</v>
       </c>
@@ -3755,7 +3739,7 @@
       <c r="F279" s="10"/>
       <c r="G279" s="5"/>
     </row>
-    <row r="280" spans="2:7" ht="30" customHeight="1">
+    <row r="280" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B280" s="20">
         <v>11</v>
       </c>
@@ -3765,7 +3749,7 @@
       <c r="F280" s="10"/>
       <c r="G280" s="5"/>
     </row>
-    <row r="281" spans="2:7" ht="30" customHeight="1">
+    <row r="281" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B281" s="20">
         <v>12</v>
       </c>
@@ -3775,7 +3759,7 @@
       <c r="F281" s="10"/>
       <c r="G281" s="5"/>
     </row>
-    <row r="282" spans="2:7" ht="30" customHeight="1">
+    <row r="282" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B282" s="20">
         <v>13</v>
       </c>
@@ -3785,7 +3769,7 @@
       <c r="F282" s="10"/>
       <c r="G282" s="5"/>
     </row>
-    <row r="283" spans="2:7" ht="30" customHeight="1">
+    <row r="283" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B283" s="20">
         <v>14</v>
       </c>
@@ -3795,7 +3779,7 @@
       <c r="F283" s="10"/>
       <c r="G283" s="5"/>
     </row>
-    <row r="284" spans="2:7" ht="30" customHeight="1">
+    <row r="284" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B284" s="20">
         <v>15</v>
       </c>
@@ -3805,7 +3789,7 @@
       <c r="F284" s="10"/>
       <c r="G284" s="5"/>
     </row>
-    <row r="285" spans="2:7" ht="30" customHeight="1">
+    <row r="285" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B285" s="20">
         <v>16</v>
       </c>
@@ -3815,7 +3799,7 @@
       <c r="F285" s="10"/>
       <c r="G285" s="5"/>
     </row>
-    <row r="286" spans="2:7" ht="30" customHeight="1">
+    <row r="286" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B286" s="20">
         <v>17</v>
       </c>
@@ -3825,7 +3809,7 @@
       <c r="F286" s="10"/>
       <c r="G286" s="5"/>
     </row>
-    <row r="287" spans="2:7" ht="30" customHeight="1">
+    <row r="287" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B287" s="20">
         <v>18</v>
       </c>
@@ -3835,7 +3819,7 @@
       <c r="F287" s="10"/>
       <c r="G287" s="5"/>
     </row>
-    <row r="288" spans="2:7" ht="30" customHeight="1">
+    <row r="288" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B288" s="20">
         <v>19</v>
       </c>
@@ -3845,7 +3829,7 @@
       <c r="F288" s="10"/>
       <c r="G288" s="5"/>
     </row>
-    <row r="289" spans="1:7" ht="30" customHeight="1">
+    <row r="289" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B289" s="20">
         <v>20</v>
       </c>
@@ -3858,12 +3842,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="290" spans="1:7" ht="30" customHeight="1">
+    <row r="290" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B290" s="19"/>
       <c r="E290" s="12"/>
       <c r="F290" s="13"/>
     </row>
-    <row r="291" spans="1:7" ht="30" customHeight="1">
+    <row r="291" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A291" s="15">
         <v>14</v>
       </c>
@@ -3873,7 +3857,7 @@
       </c>
       <c r="F291" s="9"/>
     </row>
-    <row r="292" spans="1:7" ht="30" customHeight="1">
+    <row r="292" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B292" s="20">
         <v>1</v>
       </c>
@@ -3883,7 +3867,7 @@
       <c r="F292" s="10"/>
       <c r="G292" s="5"/>
     </row>
-    <row r="293" spans="1:7" ht="30" customHeight="1">
+    <row r="293" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B293" s="20">
         <v>2</v>
       </c>
@@ -3893,7 +3877,7 @@
       <c r="F293" s="10"/>
       <c r="G293" s="5"/>
     </row>
-    <row r="294" spans="1:7" ht="30" customHeight="1">
+    <row r="294" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B294" s="20">
         <v>3</v>
       </c>
@@ -3903,7 +3887,7 @@
       <c r="F294" s="10"/>
       <c r="G294" s="5"/>
     </row>
-    <row r="295" spans="1:7" ht="30" customHeight="1">
+    <row r="295" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B295" s="20">
         <v>4</v>
       </c>
@@ -3913,7 +3897,7 @@
       <c r="F295" s="10"/>
       <c r="G295" s="5"/>
     </row>
-    <row r="296" spans="1:7" ht="30" customHeight="1">
+    <row r="296" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B296" s="20">
         <v>5</v>
       </c>
@@ -3923,7 +3907,7 @@
       <c r="F296" s="10"/>
       <c r="G296" s="5"/>
     </row>
-    <row r="297" spans="1:7" ht="30" customHeight="1">
+    <row r="297" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B297" s="20">
         <v>6</v>
       </c>
@@ -3933,7 +3917,7 @@
       <c r="F297" s="10"/>
       <c r="G297" s="5"/>
     </row>
-    <row r="298" spans="1:7" ht="30" customHeight="1">
+    <row r="298" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B298" s="20">
         <v>7</v>
       </c>
@@ -3943,7 +3927,7 @@
       <c r="F298" s="10"/>
       <c r="G298" s="5"/>
     </row>
-    <row r="299" spans="1:7" ht="30" customHeight="1">
+    <row r="299" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B299" s="20">
         <v>8</v>
       </c>
@@ -3953,7 +3937,7 @@
       <c r="F299" s="10"/>
       <c r="G299" s="5"/>
     </row>
-    <row r="300" spans="1:7" ht="30" customHeight="1">
+    <row r="300" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B300" s="20">
         <v>9</v>
       </c>
@@ -3963,7 +3947,7 @@
       <c r="F300" s="10"/>
       <c r="G300" s="5"/>
     </row>
-    <row r="301" spans="1:7" ht="30" customHeight="1">
+    <row r="301" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B301" s="20">
         <v>10</v>
       </c>
@@ -3973,7 +3957,7 @@
       <c r="F301" s="10"/>
       <c r="G301" s="5"/>
     </row>
-    <row r="302" spans="1:7" ht="30" customHeight="1">
+    <row r="302" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B302" s="20">
         <v>11</v>
       </c>
@@ -3983,7 +3967,7 @@
       <c r="F302" s="10"/>
       <c r="G302" s="5"/>
     </row>
-    <row r="303" spans="1:7" ht="30" customHeight="1">
+    <row r="303" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B303" s="20">
         <v>12</v>
       </c>
@@ -3993,7 +3977,7 @@
       <c r="F303" s="10"/>
       <c r="G303" s="5"/>
     </row>
-    <row r="304" spans="1:7" ht="30" customHeight="1">
+    <row r="304" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B304" s="20">
         <v>13</v>
       </c>
@@ -4003,7 +3987,7 @@
       <c r="F304" s="10"/>
       <c r="G304" s="5"/>
     </row>
-    <row r="305" spans="1:7" ht="30" customHeight="1">
+    <row r="305" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B305" s="20">
         <v>14</v>
       </c>
@@ -4013,7 +3997,7 @@
       <c r="F305" s="10"/>
       <c r="G305" s="5"/>
     </row>
-    <row r="306" spans="1:7" ht="30" customHeight="1">
+    <row r="306" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B306" s="20">
         <v>15</v>
       </c>
@@ -4023,7 +4007,7 @@
       <c r="F306" s="10"/>
       <c r="G306" s="5"/>
     </row>
-    <row r="307" spans="1:7" ht="30" customHeight="1">
+    <row r="307" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B307" s="20">
         <v>16</v>
       </c>
@@ -4033,7 +4017,7 @@
       <c r="F307" s="10"/>
       <c r="G307" s="5"/>
     </row>
-    <row r="308" spans="1:7" ht="30" customHeight="1">
+    <row r="308" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B308" s="20">
         <v>17</v>
       </c>
@@ -4043,7 +4027,7 @@
       <c r="F308" s="10"/>
       <c r="G308" s="5"/>
     </row>
-    <row r="309" spans="1:7" ht="30" customHeight="1">
+    <row r="309" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B309" s="20">
         <v>18</v>
       </c>
@@ -4053,7 +4037,7 @@
       <c r="F309" s="10"/>
       <c r="G309" s="5"/>
     </row>
-    <row r="310" spans="1:7" ht="30" customHeight="1">
+    <row r="310" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B310" s="20">
         <v>19</v>
       </c>
@@ -4063,7 +4047,7 @@
       <c r="F310" s="10"/>
       <c r="G310" s="5"/>
     </row>
-    <row r="311" spans="1:7" ht="30" customHeight="1">
+    <row r="311" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B311" s="20">
         <v>20</v>
       </c>
@@ -4076,12 +4060,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="312" spans="1:7" ht="30" customHeight="1">
+    <row r="312" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B312" s="19"/>
       <c r="E312" s="12"/>
       <c r="F312" s="13"/>
     </row>
-    <row r="313" spans="1:7" ht="30" customHeight="1">
+    <row r="313" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A313" s="15">
         <v>15</v>
       </c>
@@ -4091,7 +4075,7 @@
       </c>
       <c r="F313" s="9"/>
     </row>
-    <row r="314" spans="1:7" ht="30" customHeight="1">
+    <row r="314" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B314" s="20">
         <v>1</v>
       </c>
@@ -4101,7 +4085,7 @@
       <c r="F314" s="10"/>
       <c r="G314" s="5"/>
     </row>
-    <row r="315" spans="1:7" ht="30" customHeight="1">
+    <row r="315" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B315" s="20">
         <v>2</v>
       </c>
@@ -4111,7 +4095,7 @@
       <c r="F315" s="10"/>
       <c r="G315" s="5"/>
     </row>
-    <row r="316" spans="1:7" ht="30" customHeight="1">
+    <row r="316" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B316" s="20">
         <v>3</v>
       </c>
@@ -4121,7 +4105,7 @@
       <c r="F316" s="10"/>
       <c r="G316" s="5"/>
     </row>
-    <row r="317" spans="1:7" ht="30" customHeight="1">
+    <row r="317" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B317" s="20">
         <v>4</v>
       </c>
@@ -4131,7 +4115,7 @@
       <c r="F317" s="10"/>
       <c r="G317" s="5"/>
     </row>
-    <row r="318" spans="1:7" ht="30" customHeight="1">
+    <row r="318" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B318" s="20">
         <v>5</v>
       </c>
@@ -4141,7 +4125,7 @@
       <c r="F318" s="10"/>
       <c r="G318" s="5"/>
     </row>
-    <row r="319" spans="1:7" ht="30" customHeight="1">
+    <row r="319" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B319" s="20">
         <v>6</v>
       </c>
@@ -4151,7 +4135,7 @@
       <c r="F319" s="10"/>
       <c r="G319" s="5"/>
     </row>
-    <row r="320" spans="1:7" ht="30" customHeight="1">
+    <row r="320" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B320" s="20">
         <v>7</v>
       </c>
@@ -4161,7 +4145,7 @@
       <c r="F320" s="10"/>
       <c r="G320" s="5"/>
     </row>
-    <row r="321" spans="1:7" ht="30" customHeight="1">
+    <row r="321" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B321" s="20">
         <v>8</v>
       </c>
@@ -4171,7 +4155,7 @@
       <c r="F321" s="10"/>
       <c r="G321" s="5"/>
     </row>
-    <row r="322" spans="1:7" ht="30" customHeight="1">
+    <row r="322" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B322" s="20">
         <v>9</v>
       </c>
@@ -4181,7 +4165,7 @@
       <c r="F322" s="10"/>
       <c r="G322" s="5"/>
     </row>
-    <row r="323" spans="1:7" ht="30" customHeight="1">
+    <row r="323" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B323" s="20">
         <v>10</v>
       </c>
@@ -4191,7 +4175,7 @@
       <c r="F323" s="10"/>
       <c r="G323" s="5"/>
     </row>
-    <row r="324" spans="1:7" ht="30" customHeight="1">
+    <row r="324" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B324" s="20">
         <v>11</v>
       </c>
@@ -4201,7 +4185,7 @@
       <c r="F324" s="10"/>
       <c r="G324" s="5"/>
     </row>
-    <row r="325" spans="1:7" ht="30" customHeight="1">
+    <row r="325" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B325" s="20">
         <v>12</v>
       </c>
@@ -4211,7 +4195,7 @@
       <c r="F325" s="10"/>
       <c r="G325" s="5"/>
     </row>
-    <row r="326" spans="1:7" ht="30" customHeight="1">
+    <row r="326" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B326" s="20">
         <v>13</v>
       </c>
@@ -4221,7 +4205,7 @@
       <c r="F326" s="10"/>
       <c r="G326" s="5"/>
     </row>
-    <row r="327" spans="1:7" ht="30" customHeight="1">
+    <row r="327" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B327" s="20">
         <v>14</v>
       </c>
@@ -4231,7 +4215,7 @@
       <c r="F327" s="10"/>
       <c r="G327" s="5"/>
     </row>
-    <row r="328" spans="1:7" ht="30" customHeight="1">
+    <row r="328" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B328" s="20">
         <v>15</v>
       </c>
@@ -4241,7 +4225,7 @@
       <c r="F328" s="10"/>
       <c r="G328" s="5"/>
     </row>
-    <row r="329" spans="1:7" ht="30" customHeight="1">
+    <row r="329" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B329" s="20">
         <v>16</v>
       </c>
@@ -4251,7 +4235,7 @@
       <c r="F329" s="10"/>
       <c r="G329" s="5"/>
     </row>
-    <row r="330" spans="1:7" ht="30" customHeight="1">
+    <row r="330" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B330" s="20">
         <v>17</v>
       </c>
@@ -4261,7 +4245,7 @@
       <c r="F330" s="10"/>
       <c r="G330" s="5"/>
     </row>
-    <row r="331" spans="1:7" ht="30" customHeight="1">
+    <row r="331" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B331" s="20">
         <v>18</v>
       </c>
@@ -4271,7 +4255,7 @@
       <c r="F331" s="10"/>
       <c r="G331" s="5"/>
     </row>
-    <row r="332" spans="1:7" ht="30" customHeight="1">
+    <row r="332" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B332" s="20">
         <v>19</v>
       </c>
@@ -4281,7 +4265,7 @@
       <c r="F332" s="10"/>
       <c r="G332" s="5"/>
     </row>
-    <row r="333" spans="1:7" ht="30" customHeight="1">
+    <row r="333" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B333" s="20">
         <v>20</v>
       </c>
@@ -4294,12 +4278,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="334" spans="1:7" ht="30" customHeight="1">
+    <row r="334" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B334" s="19"/>
       <c r="E334" s="12"/>
       <c r="F334" s="13"/>
     </row>
-    <row r="335" spans="1:7" ht="30" customHeight="1">
+    <row r="335" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A335" s="15">
         <v>16</v>
       </c>
@@ -4309,7 +4293,7 @@
       </c>
       <c r="F335" s="9"/>
     </row>
-    <row r="336" spans="1:7" ht="30" customHeight="1">
+    <row r="336" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B336" s="20">
         <v>1</v>
       </c>
@@ -4319,7 +4303,7 @@
       <c r="F336" s="10"/>
       <c r="G336" s="5"/>
     </row>
-    <row r="337" spans="2:7" ht="30" customHeight="1">
+    <row r="337" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B337" s="20">
         <v>2</v>
       </c>
@@ -4329,7 +4313,7 @@
       <c r="F337" s="10"/>
       <c r="G337" s="5"/>
     </row>
-    <row r="338" spans="2:7" ht="30" customHeight="1">
+    <row r="338" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B338" s="20">
         <v>3</v>
       </c>
@@ -4339,7 +4323,7 @@
       <c r="F338" s="10"/>
       <c r="G338" s="5"/>
     </row>
-    <row r="339" spans="2:7" ht="30" customHeight="1">
+    <row r="339" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B339" s="20">
         <v>4</v>
       </c>
@@ -4349,7 +4333,7 @@
       <c r="F339" s="10"/>
       <c r="G339" s="5"/>
     </row>
-    <row r="340" spans="2:7" ht="30" customHeight="1">
+    <row r="340" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B340" s="20">
         <v>5</v>
       </c>
@@ -4359,7 +4343,7 @@
       <c r="F340" s="10"/>
       <c r="G340" s="5"/>
     </row>
-    <row r="341" spans="2:7" ht="30" customHeight="1">
+    <row r="341" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B341" s="20">
         <v>6</v>
       </c>
@@ -4369,7 +4353,7 @@
       <c r="F341" s="10"/>
       <c r="G341" s="5"/>
     </row>
-    <row r="342" spans="2:7" ht="30" customHeight="1">
+    <row r="342" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B342" s="20">
         <v>7</v>
       </c>
@@ -4379,7 +4363,7 @@
       <c r="F342" s="10"/>
       <c r="G342" s="5"/>
     </row>
-    <row r="343" spans="2:7" ht="30" customHeight="1">
+    <row r="343" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B343" s="20">
         <v>8</v>
       </c>
@@ -4389,7 +4373,7 @@
       <c r="F343" s="10"/>
       <c r="G343" s="5"/>
     </row>
-    <row r="344" spans="2:7" ht="30" customHeight="1">
+    <row r="344" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B344" s="20">
         <v>9</v>
       </c>
@@ -4399,7 +4383,7 @@
       <c r="F344" s="10"/>
       <c r="G344" s="5"/>
     </row>
-    <row r="345" spans="2:7" ht="30" customHeight="1">
+    <row r="345" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B345" s="20">
         <v>10</v>
       </c>
@@ -4409,7 +4393,7 @@
       <c r="F345" s="10"/>
       <c r="G345" s="5"/>
     </row>
-    <row r="346" spans="2:7" ht="30" customHeight="1">
+    <row r="346" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B346" s="20">
         <v>11</v>
       </c>
@@ -4419,7 +4403,7 @@
       <c r="F346" s="10"/>
       <c r="G346" s="5"/>
     </row>
-    <row r="347" spans="2:7" ht="30" customHeight="1">
+    <row r="347" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B347" s="20">
         <v>12</v>
       </c>
@@ -4429,7 +4413,7 @@
       <c r="F347" s="10"/>
       <c r="G347" s="5"/>
     </row>
-    <row r="348" spans="2:7" ht="30" customHeight="1">
+    <row r="348" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B348" s="20">
         <v>13</v>
       </c>
@@ -4439,7 +4423,7 @@
       <c r="F348" s="10"/>
       <c r="G348" s="5"/>
     </row>
-    <row r="349" spans="2:7" ht="30" customHeight="1">
+    <row r="349" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B349" s="20">
         <v>14</v>
       </c>
@@ -4449,7 +4433,7 @@
       <c r="F349" s="10"/>
       <c r="G349" s="5"/>
     </row>
-    <row r="350" spans="2:7" ht="30" customHeight="1">
+    <row r="350" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B350" s="20">
         <v>15</v>
       </c>
@@ -4459,7 +4443,7 @@
       <c r="F350" s="10"/>
       <c r="G350" s="5"/>
     </row>
-    <row r="351" spans="2:7" ht="30" customHeight="1">
+    <row r="351" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B351" s="20">
         <v>16</v>
       </c>
@@ -4469,7 +4453,7 @@
       <c r="F351" s="10"/>
       <c r="G351" s="5"/>
     </row>
-    <row r="352" spans="2:7" ht="30" customHeight="1">
+    <row r="352" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B352" s="20">
         <v>17</v>
       </c>
@@ -4479,7 +4463,7 @@
       <c r="F352" s="10"/>
       <c r="G352" s="5"/>
     </row>
-    <row r="353" spans="1:7" ht="30" customHeight="1">
+    <row r="353" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B353" s="20">
         <v>18</v>
       </c>
@@ -4489,7 +4473,7 @@
       <c r="F353" s="10"/>
       <c r="G353" s="5"/>
     </row>
-    <row r="354" spans="1:7" ht="30" customHeight="1">
+    <row r="354" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B354" s="20">
         <v>19</v>
       </c>
@@ -4499,7 +4483,7 @@
       <c r="F354" s="10"/>
       <c r="G354" s="5"/>
     </row>
-    <row r="355" spans="1:7" ht="30" customHeight="1">
+    <row r="355" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B355" s="20">
         <v>20</v>
       </c>
@@ -4512,12 +4496,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="356" spans="1:7" ht="30" customHeight="1">
+    <row r="356" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B356" s="19"/>
       <c r="E356" s="12"/>
       <c r="F356" s="13"/>
     </row>
-    <row r="357" spans="1:7" ht="30" customHeight="1">
+    <row r="357" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A357" s="15">
         <v>17</v>
       </c>
@@ -4527,7 +4511,7 @@
       </c>
       <c r="F357" s="9"/>
     </row>
-    <row r="358" spans="1:7" ht="30" customHeight="1">
+    <row r="358" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B358" s="20">
         <v>1</v>
       </c>
@@ -4537,7 +4521,7 @@
       <c r="F358" s="10"/>
       <c r="G358" s="5"/>
     </row>
-    <row r="359" spans="1:7" ht="30" customHeight="1">
+    <row r="359" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B359" s="20">
         <v>2</v>
       </c>
@@ -4547,7 +4531,7 @@
       <c r="F359" s="10"/>
       <c r="G359" s="5"/>
     </row>
-    <row r="360" spans="1:7" ht="30" customHeight="1">
+    <row r="360" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B360" s="20">
         <v>3</v>
       </c>
@@ -4557,7 +4541,7 @@
       <c r="F360" s="10"/>
       <c r="G360" s="5"/>
     </row>
-    <row r="361" spans="1:7" ht="30" customHeight="1">
+    <row r="361" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B361" s="20">
         <v>4</v>
       </c>
@@ -4567,7 +4551,7 @@
       <c r="F361" s="10"/>
       <c r="G361" s="5"/>
     </row>
-    <row r="362" spans="1:7" ht="30" customHeight="1">
+    <row r="362" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B362" s="20">
         <v>5</v>
       </c>
@@ -4577,7 +4561,7 @@
       <c r="F362" s="10"/>
       <c r="G362" s="5"/>
     </row>
-    <row r="363" spans="1:7" ht="30" customHeight="1">
+    <row r="363" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B363" s="20">
         <v>6</v>
       </c>
@@ -4587,7 +4571,7 @@
       <c r="F363" s="10"/>
       <c r="G363" s="5"/>
     </row>
-    <row r="364" spans="1:7" ht="30" customHeight="1">
+    <row r="364" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B364" s="20">
         <v>7</v>
       </c>
@@ -4597,7 +4581,7 @@
       <c r="F364" s="10"/>
       <c r="G364" s="5"/>
     </row>
-    <row r="365" spans="1:7" ht="30" customHeight="1">
+    <row r="365" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B365" s="20">
         <v>8</v>
       </c>
@@ -4607,7 +4591,7 @@
       <c r="F365" s="10"/>
       <c r="G365" s="5"/>
     </row>
-    <row r="366" spans="1:7" ht="30" customHeight="1">
+    <row r="366" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B366" s="20">
         <v>9</v>
       </c>
@@ -4617,7 +4601,7 @@
       <c r="F366" s="10"/>
       <c r="G366" s="5"/>
     </row>
-    <row r="367" spans="1:7" ht="30" customHeight="1">
+    <row r="367" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B367" s="20">
         <v>10</v>
       </c>
@@ -4627,7 +4611,7 @@
       <c r="F367" s="10"/>
       <c r="G367" s="5"/>
     </row>
-    <row r="368" spans="1:7" ht="30" customHeight="1">
+    <row r="368" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B368" s="20">
         <v>11</v>
       </c>
@@ -4637,7 +4621,7 @@
       <c r="F368" s="10"/>
       <c r="G368" s="5"/>
     </row>
-    <row r="369" spans="1:7" ht="30" customHeight="1">
+    <row r="369" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B369" s="20">
         <v>12</v>
       </c>
@@ -4647,7 +4631,7 @@
       <c r="F369" s="10"/>
       <c r="G369" s="5"/>
     </row>
-    <row r="370" spans="1:7" ht="30" customHeight="1">
+    <row r="370" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B370" s="20">
         <v>13</v>
       </c>
@@ -4657,7 +4641,7 @@
       <c r="F370" s="10"/>
       <c r="G370" s="5"/>
     </row>
-    <row r="371" spans="1:7" ht="30" customHeight="1">
+    <row r="371" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B371" s="20">
         <v>14</v>
       </c>
@@ -4667,7 +4651,7 @@
       <c r="F371" s="10"/>
       <c r="G371" s="5"/>
     </row>
-    <row r="372" spans="1:7" ht="30" customHeight="1">
+    <row r="372" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B372" s="20">
         <v>15</v>
       </c>
@@ -4677,7 +4661,7 @@
       <c r="F372" s="10"/>
       <c r="G372" s="5"/>
     </row>
-    <row r="373" spans="1:7" ht="30" customHeight="1">
+    <row r="373" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B373" s="20">
         <v>16</v>
       </c>
@@ -4687,7 +4671,7 @@
       <c r="F373" s="10"/>
       <c r="G373" s="5"/>
     </row>
-    <row r="374" spans="1:7" ht="30" customHeight="1">
+    <row r="374" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B374" s="20">
         <v>17</v>
       </c>
@@ -4697,7 +4681,7 @@
       <c r="F374" s="10"/>
       <c r="G374" s="5"/>
     </row>
-    <row r="375" spans="1:7" ht="30" customHeight="1">
+    <row r="375" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B375" s="20">
         <v>18</v>
       </c>
@@ -4707,7 +4691,7 @@
       <c r="F375" s="10"/>
       <c r="G375" s="5"/>
     </row>
-    <row r="376" spans="1:7" ht="30" customHeight="1">
+    <row r="376" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B376" s="20">
         <v>19</v>
       </c>
@@ -4717,7 +4701,7 @@
       <c r="F376" s="10"/>
       <c r="G376" s="5"/>
     </row>
-    <row r="377" spans="1:7" ht="30" customHeight="1">
+    <row r="377" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B377" s="20">
         <v>20</v>
       </c>
@@ -4730,12 +4714,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="378" spans="1:7" ht="30" customHeight="1">
+    <row r="378" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B378" s="19"/>
       <c r="E378" s="12"/>
       <c r="F378" s="13"/>
     </row>
-    <row r="379" spans="1:7" ht="30" customHeight="1">
+    <row r="379" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A379" s="15">
         <v>18</v>
       </c>
@@ -4745,7 +4729,7 @@
       </c>
       <c r="F379" s="9"/>
     </row>
-    <row r="380" spans="1:7" ht="30" customHeight="1">
+    <row r="380" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B380" s="20">
         <v>1</v>
       </c>
@@ -4755,7 +4739,7 @@
       <c r="F380" s="10"/>
       <c r="G380" s="5"/>
     </row>
-    <row r="381" spans="1:7" ht="30" customHeight="1">
+    <row r="381" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B381" s="20">
         <v>2</v>
       </c>
@@ -4765,7 +4749,7 @@
       <c r="F381" s="10"/>
       <c r="G381" s="5"/>
     </row>
-    <row r="382" spans="1:7" ht="30" customHeight="1">
+    <row r="382" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B382" s="20">
         <v>3</v>
       </c>
@@ -4775,7 +4759,7 @@
       <c r="F382" s="10"/>
       <c r="G382" s="5"/>
     </row>
-    <row r="383" spans="1:7" ht="30" customHeight="1">
+    <row r="383" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B383" s="20">
         <v>4</v>
       </c>
@@ -4785,7 +4769,7 @@
       <c r="F383" s="10"/>
       <c r="G383" s="5"/>
     </row>
-    <row r="384" spans="1:7" ht="30" customHeight="1">
+    <row r="384" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B384" s="20">
         <v>5</v>
       </c>
@@ -4795,7 +4779,7 @@
       <c r="F384" s="10"/>
       <c r="G384" s="5"/>
     </row>
-    <row r="385" spans="2:7" ht="30" customHeight="1">
+    <row r="385" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B385" s="20">
         <v>6</v>
       </c>
@@ -4805,7 +4789,7 @@
       <c r="F385" s="10"/>
       <c r="G385" s="5"/>
     </row>
-    <row r="386" spans="2:7" ht="30" customHeight="1">
+    <row r="386" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B386" s="20">
         <v>7</v>
       </c>
@@ -4815,7 +4799,7 @@
       <c r="F386" s="10"/>
       <c r="G386" s="5"/>
     </row>
-    <row r="387" spans="2:7" ht="30" customHeight="1">
+    <row r="387" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B387" s="20">
         <v>8</v>
       </c>
@@ -4825,7 +4809,7 @@
       <c r="F387" s="10"/>
       <c r="G387" s="5"/>
     </row>
-    <row r="388" spans="2:7" ht="30" customHeight="1">
+    <row r="388" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B388" s="20">
         <v>9</v>
       </c>
@@ -4835,7 +4819,7 @@
       <c r="F388" s="10"/>
       <c r="G388" s="5"/>
     </row>
-    <row r="389" spans="2:7" ht="30" customHeight="1">
+    <row r="389" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B389" s="20">
         <v>10</v>
       </c>
@@ -4845,7 +4829,7 @@
       <c r="F389" s="10"/>
       <c r="G389" s="5"/>
     </row>
-    <row r="390" spans="2:7" ht="30" customHeight="1">
+    <row r="390" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B390" s="20">
         <v>11</v>
       </c>
@@ -4855,7 +4839,7 @@
       <c r="F390" s="10"/>
       <c r="G390" s="5"/>
     </row>
-    <row r="391" spans="2:7" ht="30" customHeight="1">
+    <row r="391" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B391" s="20">
         <v>12</v>
       </c>
@@ -4865,7 +4849,7 @@
       <c r="F391" s="10"/>
       <c r="G391" s="5"/>
     </row>
-    <row r="392" spans="2:7" ht="30" customHeight="1">
+    <row r="392" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B392" s="20">
         <v>13</v>
       </c>
@@ -4875,7 +4859,7 @@
       <c r="F392" s="10"/>
       <c r="G392" s="5"/>
     </row>
-    <row r="393" spans="2:7" ht="30" customHeight="1">
+    <row r="393" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B393" s="20">
         <v>14</v>
       </c>
@@ -4885,7 +4869,7 @@
       <c r="F393" s="10"/>
       <c r="G393" s="5"/>
     </row>
-    <row r="394" spans="2:7" ht="30" customHeight="1">
+    <row r="394" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B394" s="20">
         <v>15</v>
       </c>
@@ -4895,7 +4879,7 @@
       <c r="F394" s="10"/>
       <c r="G394" s="5"/>
     </row>
-    <row r="395" spans="2:7" ht="30" customHeight="1">
+    <row r="395" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B395" s="20">
         <v>16</v>
       </c>
@@ -4905,7 +4889,7 @@
       <c r="F395" s="10"/>
       <c r="G395" s="5"/>
     </row>
-    <row r="396" spans="2:7" ht="30" customHeight="1">
+    <row r="396" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B396" s="20">
         <v>17</v>
       </c>
@@ -4915,7 +4899,7 @@
       <c r="F396" s="10"/>
       <c r="G396" s="5"/>
     </row>
-    <row r="397" spans="2:7" ht="30" customHeight="1">
+    <row r="397" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B397" s="20">
         <v>18</v>
       </c>
@@ -4925,7 +4909,7 @@
       <c r="F397" s="10"/>
       <c r="G397" s="5"/>
     </row>
-    <row r="398" spans="2:7" ht="30" customHeight="1">
+    <row r="398" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B398" s="20">
         <v>19</v>
       </c>
@@ -4935,7 +4919,7 @@
       <c r="F398" s="10"/>
       <c r="G398" s="5"/>
     </row>
-    <row r="399" spans="2:7" ht="30" customHeight="1">
+    <row r="399" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B399" s="20">
         <v>20</v>
       </c>
@@ -4948,12 +4932,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="400" spans="2:7" ht="30" customHeight="1">
+    <row r="400" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B400" s="19"/>
       <c r="E400" s="12"/>
       <c r="F400" s="13"/>
     </row>
-    <row r="401" spans="1:7" ht="30" customHeight="1">
+    <row r="401" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A401" s="15">
         <v>19</v>
       </c>
@@ -4963,7 +4947,7 @@
       </c>
       <c r="F401" s="9"/>
     </row>
-    <row r="402" spans="1:7" ht="30" customHeight="1">
+    <row r="402" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B402" s="20">
         <v>1</v>
       </c>
@@ -4973,7 +4957,7 @@
       <c r="F402" s="10"/>
       <c r="G402" s="5"/>
     </row>
-    <row r="403" spans="1:7" ht="30" customHeight="1">
+    <row r="403" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B403" s="20">
         <v>2</v>
       </c>
@@ -4983,7 +4967,7 @@
       <c r="F403" s="10"/>
       <c r="G403" s="5"/>
     </row>
-    <row r="404" spans="1:7" ht="30" customHeight="1">
+    <row r="404" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B404" s="20">
         <v>3</v>
       </c>
@@ -4993,7 +4977,7 @@
       <c r="F404" s="10"/>
       <c r="G404" s="5"/>
     </row>
-    <row r="405" spans="1:7" ht="30" customHeight="1">
+    <row r="405" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B405" s="20">
         <v>4</v>
       </c>
@@ -5003,7 +4987,7 @@
       <c r="F405" s="10"/>
       <c r="G405" s="5"/>
     </row>
-    <row r="406" spans="1:7" ht="30" customHeight="1">
+    <row r="406" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B406" s="20">
         <v>5</v>
       </c>
@@ -5013,7 +4997,7 @@
       <c r="F406" s="10"/>
       <c r="G406" s="5"/>
     </row>
-    <row r="407" spans="1:7" ht="30" customHeight="1">
+    <row r="407" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B407" s="20">
         <v>6</v>
       </c>
@@ -5023,7 +5007,7 @@
       <c r="F407" s="10"/>
       <c r="G407" s="5"/>
     </row>
-    <row r="408" spans="1:7" ht="30" customHeight="1">
+    <row r="408" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B408" s="20">
         <v>7</v>
       </c>
@@ -5033,7 +5017,7 @@
       <c r="F408" s="10"/>
       <c r="G408" s="5"/>
     </row>
-    <row r="409" spans="1:7" ht="30" customHeight="1">
+    <row r="409" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B409" s="20">
         <v>8</v>
       </c>
@@ -5043,7 +5027,7 @@
       <c r="F409" s="10"/>
       <c r="G409" s="5"/>
     </row>
-    <row r="410" spans="1:7" ht="30" customHeight="1">
+    <row r="410" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B410" s="20">
         <v>9</v>
       </c>
@@ -5053,7 +5037,7 @@
       <c r="F410" s="10"/>
       <c r="G410" s="5"/>
     </row>
-    <row r="411" spans="1:7" ht="30" customHeight="1">
+    <row r="411" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B411" s="20">
         <v>10</v>
       </c>
@@ -5063,7 +5047,7 @@
       <c r="F411" s="10"/>
       <c r="G411" s="5"/>
     </row>
-    <row r="412" spans="1:7" ht="30" customHeight="1">
+    <row r="412" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B412" s="20">
         <v>11</v>
       </c>
@@ -5073,7 +5057,7 @@
       <c r="F412" s="10"/>
       <c r="G412" s="5"/>
     </row>
-    <row r="413" spans="1:7" ht="30" customHeight="1">
+    <row r="413" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B413" s="20">
         <v>12</v>
       </c>
@@ -5083,7 +5067,7 @@
       <c r="F413" s="10"/>
       <c r="G413" s="5"/>
     </row>
-    <row r="414" spans="1:7" ht="30" customHeight="1">
+    <row r="414" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B414" s="20">
         <v>13</v>
       </c>
@@ -5093,7 +5077,7 @@
       <c r="F414" s="10"/>
       <c r="G414" s="5"/>
     </row>
-    <row r="415" spans="1:7" ht="30" customHeight="1">
+    <row r="415" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B415" s="20">
         <v>14</v>
       </c>
@@ -5103,7 +5087,7 @@
       <c r="F415" s="10"/>
       <c r="G415" s="5"/>
     </row>
-    <row r="416" spans="1:7" ht="30" customHeight="1">
+    <row r="416" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B416" s="20">
         <v>15</v>
       </c>
@@ -5113,7 +5097,7 @@
       <c r="F416" s="10"/>
       <c r="G416" s="5"/>
     </row>
-    <row r="417" spans="1:7" ht="30" customHeight="1">
+    <row r="417" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B417" s="20">
         <v>16</v>
       </c>
@@ -5123,7 +5107,7 @@
       <c r="F417" s="10"/>
       <c r="G417" s="5"/>
     </row>
-    <row r="418" spans="1:7" ht="30" customHeight="1">
+    <row r="418" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B418" s="20">
         <v>17</v>
       </c>
@@ -5133,7 +5117,7 @@
       <c r="F418" s="10"/>
       <c r="G418" s="5"/>
     </row>
-    <row r="419" spans="1:7" ht="30" customHeight="1">
+    <row r="419" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B419" s="20">
         <v>18</v>
       </c>
@@ -5143,7 +5127,7 @@
       <c r="F419" s="10"/>
       <c r="G419" s="5"/>
     </row>
-    <row r="420" spans="1:7" ht="30" customHeight="1">
+    <row r="420" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B420" s="20">
         <v>19</v>
       </c>
@@ -5153,7 +5137,7 @@
       <c r="F420" s="10"/>
       <c r="G420" s="5"/>
     </row>
-    <row r="421" spans="1:7" ht="30" customHeight="1">
+    <row r="421" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B421" s="20">
         <v>20</v>
       </c>
@@ -5166,12 +5150,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="422" spans="1:7" ht="30" customHeight="1">
+    <row r="422" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B422" s="19"/>
       <c r="E422" s="12"/>
       <c r="F422" s="13"/>
     </row>
-    <row r="423" spans="1:7" ht="30" customHeight="1">
+    <row r="423" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A423" s="15">
         <v>20</v>
       </c>
@@ -5181,7 +5165,7 @@
       </c>
       <c r="F423" s="9"/>
     </row>
-    <row r="424" spans="1:7" ht="30" customHeight="1">
+    <row r="424" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B424" s="20">
         <v>1</v>
       </c>
@@ -5191,7 +5175,7 @@
       <c r="F424" s="10"/>
       <c r="G424" s="5"/>
     </row>
-    <row r="425" spans="1:7" ht="30" customHeight="1">
+    <row r="425" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B425" s="20">
         <v>2</v>
       </c>
@@ -5201,7 +5185,7 @@
       <c r="F425" s="10"/>
       <c r="G425" s="5"/>
     </row>
-    <row r="426" spans="1:7" ht="30" customHeight="1">
+    <row r="426" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B426" s="20">
         <v>3</v>
       </c>
@@ -5211,7 +5195,7 @@
       <c r="F426" s="10"/>
       <c r="G426" s="5"/>
     </row>
-    <row r="427" spans="1:7" ht="30" customHeight="1">
+    <row r="427" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B427" s="20">
         <v>4</v>
       </c>
@@ -5221,7 +5205,7 @@
       <c r="F427" s="10"/>
       <c r="G427" s="5"/>
     </row>
-    <row r="428" spans="1:7" ht="30" customHeight="1">
+    <row r="428" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B428" s="20">
         <v>5</v>
       </c>
@@ -5231,7 +5215,7 @@
       <c r="F428" s="10"/>
       <c r="G428" s="5"/>
     </row>
-    <row r="429" spans="1:7" ht="30" customHeight="1">
+    <row r="429" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B429" s="20">
         <v>6</v>
       </c>
@@ -5241,7 +5225,7 @@
       <c r="F429" s="10"/>
       <c r="G429" s="5"/>
     </row>
-    <row r="430" spans="1:7" ht="30" customHeight="1">
+    <row r="430" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B430" s="20">
         <v>7</v>
       </c>
@@ -5251,7 +5235,7 @@
       <c r="F430" s="10"/>
       <c r="G430" s="5"/>
     </row>
-    <row r="431" spans="1:7" ht="30" customHeight="1">
+    <row r="431" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B431" s="20">
         <v>8</v>
       </c>
@@ -5261,7 +5245,7 @@
       <c r="F431" s="10"/>
       <c r="G431" s="5"/>
     </row>
-    <row r="432" spans="1:7" ht="30" customHeight="1">
+    <row r="432" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B432" s="20">
         <v>9</v>
       </c>
@@ -5271,7 +5255,7 @@
       <c r="F432" s="10"/>
       <c r="G432" s="5"/>
     </row>
-    <row r="433" spans="2:7" ht="30" customHeight="1">
+    <row r="433" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B433" s="20">
         <v>10</v>
       </c>
@@ -5281,7 +5265,7 @@
       <c r="F433" s="10"/>
       <c r="G433" s="5"/>
     </row>
-    <row r="434" spans="2:7" ht="30" customHeight="1">
+    <row r="434" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B434" s="20">
         <v>11</v>
       </c>
@@ -5291,7 +5275,7 @@
       <c r="F434" s="10"/>
       <c r="G434" s="5"/>
     </row>
-    <row r="435" spans="2:7" ht="30" customHeight="1">
+    <row r="435" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B435" s="20">
         <v>12</v>
       </c>
@@ -5301,7 +5285,7 @@
       <c r="F435" s="10"/>
       <c r="G435" s="5"/>
     </row>
-    <row r="436" spans="2:7" ht="30" customHeight="1">
+    <row r="436" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B436" s="20">
         <v>13</v>
       </c>
@@ -5311,7 +5295,7 @@
       <c r="F436" s="10"/>
       <c r="G436" s="5"/>
     </row>
-    <row r="437" spans="2:7" ht="30" customHeight="1">
+    <row r="437" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B437" s="20">
         <v>14</v>
       </c>
@@ -5321,7 +5305,7 @@
       <c r="F437" s="10"/>
       <c r="G437" s="5"/>
     </row>
-    <row r="438" spans="2:7" ht="30" customHeight="1">
+    <row r="438" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B438" s="20">
         <v>15</v>
       </c>
@@ -5331,7 +5315,7 @@
       <c r="F438" s="10"/>
       <c r="G438" s="5"/>
     </row>
-    <row r="439" spans="2:7" ht="30" customHeight="1">
+    <row r="439" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B439" s="20">
         <v>16</v>
       </c>
@@ -5341,7 +5325,7 @@
       <c r="F439" s="10"/>
       <c r="G439" s="5"/>
     </row>
-    <row r="440" spans="2:7" ht="30" customHeight="1">
+    <row r="440" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B440" s="20">
         <v>17</v>
       </c>
@@ -5351,7 +5335,7 @@
       <c r="F440" s="10"/>
       <c r="G440" s="5"/>
     </row>
-    <row r="441" spans="2:7" ht="30" customHeight="1">
+    <row r="441" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B441" s="20">
         <v>18</v>
       </c>
@@ -5361,7 +5345,7 @@
       <c r="F441" s="10"/>
       <c r="G441" s="5"/>
     </row>
-    <row r="442" spans="2:7" ht="30" customHeight="1">
+    <row r="442" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B442" s="20">
         <v>19</v>
       </c>
@@ -5371,7 +5355,7 @@
       <c r="F442" s="10"/>
       <c r="G442" s="5"/>
     </row>
-    <row r="443" spans="2:7" ht="30" customHeight="1">
+    <row r="443" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B443" s="20">
         <v>20</v>
       </c>
@@ -5384,12 +5368,12 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="444" spans="2:7" ht="15.6">
+    <row r="444" spans="2:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B444" s="19"/>
       <c r="E444" s="12"/>
       <c r="F444" s="13"/>
     </row>
-    <row r="445" spans="2:7">
+    <row r="445" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C445" s="11" t="s">
         <v>8</v>
       </c>
@@ -5408,6 +5392,7 @@
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9d258917-277f-42cd-a3cd-14c4e9ee58bc}" enabled="1" method="Standard" siteId="{38ae3bcd-9579-4fd4-adda-b42e1495d55a}" contentBits="0" removed="0"/>
   <clbl:label id="{f0785fb4-7cd3-40c0-8122-f25147720244}" enabled="1" method="Standard" siteId="{3619ea90-fa6e-40bf-aa11-2d4a18ad7689}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>